<commit_message>
Phone/short-screen hero, compact report actions, dark highlight, README, more layout tests
</commit_message>
<xml_diff>
--- a/public/samples/arjun-icici.xlsx
+++ b/public/samples/arjun-icici.xlsx
@@ -459,16 +459,16 @@
         <v>-</v>
       </c>
       <c r="E7" t="str">
-        <v>UPI/641781576746/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/209252313850/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F7" t="str">
-        <v>551.00</v>
+        <v>291.00</v>
       </c>
       <c r="G7" t="str">
         <v>0.00</v>
       </c>
       <c r="H7" t="str">
-        <v>23259.40</v>
+        <v>23519.40</v>
       </c>
     </row>
     <row r="8">
@@ -476,25 +476,25 @@
         <v>2</v>
       </c>
       <c r="B8" t="str">
-        <v>02/07/2026</v>
+        <v>01/07/2026</v>
       </c>
       <c r="C8" t="str">
-        <v>02/07/2026</v>
+        <v>01/07/2026</v>
       </c>
       <c r="D8" t="str">
         <v>-</v>
       </c>
       <c r="E8" t="str">
-        <v>UPI/489062099414/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
+        <v>UPI/177777933212/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F8" t="str">
-        <v>1999.00</v>
+        <v>554.00</v>
       </c>
       <c r="G8" t="str">
         <v>0.00</v>
       </c>
       <c r="H8" t="str">
-        <v>21260.40</v>
+        <v>22965.40</v>
       </c>
     </row>
     <row r="9">
@@ -511,16 +511,16 @@
         <v>-</v>
       </c>
       <c r="E9" t="str">
-        <v>UPI/452856088965/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/489062099414/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
       </c>
       <c r="F9" t="str">
-        <v>567.00</v>
+        <v>1999.00</v>
       </c>
       <c r="G9" t="str">
         <v>0.00</v>
       </c>
       <c r="H9" t="str">
-        <v>20693.40</v>
+        <v>20966.40</v>
       </c>
     </row>
     <row r="10">
@@ -537,16 +537,16 @@
         <v>-</v>
       </c>
       <c r="E10" t="str">
-        <v>UPI/711973269004/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/715035672136/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F10" t="str">
-        <v>203.00</v>
+        <v>192.00</v>
       </c>
       <c r="G10" t="str">
         <v>0.00</v>
       </c>
       <c r="H10" t="str">
-        <v>20490.40</v>
+        <v>20774.40</v>
       </c>
     </row>
     <row r="11">
@@ -554,25 +554,25 @@
         <v>5</v>
       </c>
       <c r="B11" t="str">
-        <v>02/07/2026</v>
+        <v>03/07/2026</v>
       </c>
       <c r="C11" t="str">
-        <v>02/07/2026</v>
+        <v>03/07/2026</v>
       </c>
       <c r="D11" t="str">
         <v>-</v>
       </c>
       <c r="E11" t="str">
-        <v>UPI/729702782281/PUNE PRINTS/9781855701@paytm/HDFC BANK</v>
+        <v>UPI/502326153567/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F11" t="str">
-        <v>116.00</v>
+        <v>1675.28</v>
       </c>
       <c r="G11" t="str">
         <v>0.00</v>
       </c>
       <c r="H11" t="str">
-        <v>20374.40</v>
+        <v>19099.12</v>
       </c>
     </row>
     <row r="12">
@@ -589,16 +589,16 @@
         <v>-</v>
       </c>
       <c r="E12" t="str">
-        <v>UPI/502326153567/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
+        <v>UPI/711973269004/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F12" t="str">
-        <v>1675.28</v>
+        <v>647.00</v>
       </c>
       <c r="G12" t="str">
         <v>0.00</v>
       </c>
       <c r="H12" t="str">
-        <v>18699.12</v>
+        <v>18452.12</v>
       </c>
     </row>
     <row r="13">
@@ -606,25 +606,25 @@
         <v>7</v>
       </c>
       <c r="B13" t="str">
-        <v>03/07/2026</v>
+        <v>04/07/2026</v>
       </c>
       <c r="C13" t="str">
-        <v>03/07/2026</v>
+        <v>04/07/2026</v>
       </c>
       <c r="D13" t="str">
         <v>-</v>
       </c>
       <c r="E13" t="str">
-        <v>UPI/522146815061/DMART/grocery@ybl/HDFC BANK</v>
+        <v>NEFT-N186260412345-BRIGHTLOOP DESIGN LLP-INV 0712</v>
       </c>
       <c r="F13" t="str">
-        <v>2050.00</v>
+        <v>0.00</v>
       </c>
       <c r="G13" t="str">
-        <v>0.00</v>
+        <v>68000.00</v>
       </c>
       <c r="H13" t="str">
-        <v>16649.12</v>
+        <v>86452.12</v>
       </c>
     </row>
     <row r="14">
@@ -641,16 +641,16 @@
         <v>-</v>
       </c>
       <c r="E14" t="str">
-        <v>NEFT-N186260412345-BRIGHTLOOP DESIGN LLP-INV 0712</v>
+        <v>UPI/524279777449/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F14" t="str">
-        <v>0.00</v>
+        <v>219.00</v>
       </c>
       <c r="G14" t="str">
-        <v>68000.00</v>
+        <v>0.00</v>
       </c>
       <c r="H14" t="str">
-        <v>84649.12</v>
+        <v>86233.12</v>
       </c>
     </row>
     <row r="15">
@@ -658,25 +658,25 @@
         <v>9</v>
       </c>
       <c r="B15" t="str">
-        <v>04/07/2026</v>
+        <v>05/07/2026</v>
       </c>
       <c r="C15" t="str">
-        <v>04/07/2026</v>
+        <v>05/07/2026</v>
       </c>
       <c r="D15" t="str">
         <v>-</v>
       </c>
       <c r="E15" t="str">
-        <v>UPI/398779632966/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>MMT/IMPS/411219905922/Rent Jul/Meera Kulkarni/HDFC0001234</v>
       </c>
       <c r="F15" t="str">
-        <v>268.00</v>
+        <v>18500.00</v>
       </c>
       <c r="G15" t="str">
         <v>0.00</v>
       </c>
       <c r="H15" t="str">
-        <v>84381.12</v>
+        <v>67733.12</v>
       </c>
     </row>
     <row r="16">
@@ -693,16 +693,16 @@
         <v>-</v>
       </c>
       <c r="E16" t="str">
-        <v>MMT/IMPS/411219905922/Rent Jul/Meera Kulkarni/HDFC0001234</v>
+        <v>UPI/602061258722/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F16" t="str">
-        <v>18500.00</v>
+        <v>380.00</v>
       </c>
       <c r="G16" t="str">
         <v>0.00</v>
       </c>
       <c r="H16" t="str">
-        <v>65881.12</v>
+        <v>67353.12</v>
       </c>
     </row>
     <row r="17">
@@ -728,7 +728,7 @@
         <v>0.00</v>
       </c>
       <c r="H17" t="str">
-        <v>65001.12</v>
+        <v>66473.12</v>
       </c>
     </row>
     <row r="18">
@@ -745,16 +745,16 @@
         <v>-</v>
       </c>
       <c r="E18" t="str">
-        <v>UPI/884662960260/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/688856796664/VAISHALI CAFE/9724225839@paytm/HDFC BANK</v>
       </c>
       <c r="F18" t="str">
-        <v>374.00</v>
+        <v>44.00</v>
       </c>
       <c r="G18" t="str">
         <v>0.00</v>
       </c>
       <c r="H18" t="str">
-        <v>64627.12</v>
+        <v>66429.12</v>
       </c>
     </row>
     <row r="19">
@@ -762,25 +762,25 @@
         <v>13</v>
       </c>
       <c r="B19" t="str">
-        <v>07/07/2026</v>
+        <v>06/07/2026</v>
       </c>
       <c r="C19" t="str">
-        <v>07/07/2026</v>
+        <v>06/07/2026</v>
       </c>
       <c r="D19" t="str">
         <v>-</v>
       </c>
       <c r="E19" t="str">
-        <v>UPI/519787674141/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/980201849364/VAISHALI CAFE/9787184773@paytm/HDFC BANK</v>
       </c>
       <c r="F19" t="str">
-        <v>491.00</v>
+        <v>153.00</v>
       </c>
       <c r="G19" t="str">
         <v>0.00</v>
       </c>
       <c r="H19" t="str">
-        <v>64136.12</v>
+        <v>66276.12</v>
       </c>
     </row>
     <row r="20">
@@ -797,16 +797,16 @@
         <v>-</v>
       </c>
       <c r="E20" t="str">
-        <v>UPI/485184686328/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/594705817033/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F20" t="str">
-        <v>138.00</v>
+        <v>414.00</v>
       </c>
       <c r="G20" t="str">
         <v>0.00</v>
       </c>
       <c r="H20" t="str">
-        <v>63998.12</v>
+        <v>65862.12</v>
       </c>
     </row>
     <row r="21">
@@ -814,25 +814,25 @@
         <v>15</v>
       </c>
       <c r="B21" t="str">
-        <v>08/07/2026</v>
+        <v>07/07/2026</v>
       </c>
       <c r="C21" t="str">
-        <v>08/07/2026</v>
+        <v>07/07/2026</v>
       </c>
       <c r="D21" t="str">
         <v>-</v>
       </c>
       <c r="E21" t="str">
-        <v>UPI/444147536531/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
+        <v>UPI/692922910070/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F21" t="str">
-        <v>1567.00</v>
+        <v>594.00</v>
       </c>
       <c r="G21" t="str">
         <v>0.00</v>
       </c>
       <c r="H21" t="str">
-        <v>62431.12</v>
+        <v>65268.12</v>
       </c>
     </row>
     <row r="22">
@@ -849,16 +849,16 @@
         <v>-</v>
       </c>
       <c r="E22" t="str">
-        <v>UPI/857678293040/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/444147536531/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
       </c>
       <c r="F22" t="str">
-        <v>207.00</v>
+        <v>1567.00</v>
       </c>
       <c r="G22" t="str">
         <v>0.00</v>
       </c>
       <c r="H22" t="str">
-        <v>62224.12</v>
+        <v>63701.12</v>
       </c>
     </row>
     <row r="23">
@@ -866,25 +866,25 @@
         <v>17</v>
       </c>
       <c r="B23" t="str">
-        <v>08/07/2026</v>
+        <v>09/07/2026</v>
       </c>
       <c r="C23" t="str">
-        <v>08/07/2026</v>
+        <v>09/07/2026</v>
       </c>
       <c r="D23" t="str">
         <v>-</v>
       </c>
       <c r="E23" t="str">
-        <v>UPI/911075336905/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/672030546190/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F23" t="str">
-        <v>656.00</v>
+        <v>394.00</v>
       </c>
       <c r="G23" t="str">
         <v>0.00</v>
       </c>
       <c r="H23" t="str">
-        <v>61568.12</v>
+        <v>63307.12</v>
       </c>
     </row>
     <row r="24">
@@ -892,25 +892,25 @@
         <v>18</v>
       </c>
       <c r="B24" t="str">
-        <v>08/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="C24" t="str">
-        <v>08/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="D24" t="str">
         <v>-</v>
       </c>
       <c r="E24" t="str">
-        <v>UPI/177777933212/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/529038106766/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
       </c>
       <c r="F24" t="str">
-        <v>554.00</v>
+        <v>119.00</v>
       </c>
       <c r="G24" t="str">
         <v>0.00</v>
       </c>
       <c r="H24" t="str">
-        <v>61014.12</v>
+        <v>63188.12</v>
       </c>
     </row>
     <row r="25">
@@ -918,25 +918,25 @@
         <v>19</v>
       </c>
       <c r="B25" t="str">
-        <v>08/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="C25" t="str">
-        <v>08/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="D25" t="str">
         <v>-</v>
       </c>
       <c r="E25" t="str">
-        <v>UPI/579760455572/VAISHALI CAFE/9735390861@paytm/HDFC BANK</v>
+        <v>UPI/187253396678/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F25" t="str">
-        <v>185.00</v>
+        <v>630.00</v>
       </c>
       <c r="G25" t="str">
         <v>0.00</v>
       </c>
       <c r="H25" t="str">
-        <v>60829.12</v>
+        <v>62558.12</v>
       </c>
     </row>
     <row r="26">
@@ -944,25 +944,25 @@
         <v>20</v>
       </c>
       <c r="B26" t="str">
-        <v>09/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="C26" t="str">
-        <v>09/07/2026</v>
+        <v>10/07/2026</v>
       </c>
       <c r="D26" t="str">
         <v>-</v>
       </c>
       <c r="E26" t="str">
-        <v>UPI/648821998643/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/736261566611/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F26" t="str">
-        <v>231.00</v>
+        <v>1701.00</v>
       </c>
       <c r="G26" t="str">
         <v>0.00</v>
       </c>
       <c r="H26" t="str">
-        <v>60598.12</v>
+        <v>60857.12</v>
       </c>
     </row>
     <row r="27">
@@ -970,25 +970,25 @@
         <v>21</v>
       </c>
       <c r="B27" t="str">
-        <v>09/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="C27" t="str">
-        <v>09/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="D27" t="str">
         <v>-</v>
       </c>
       <c r="E27" t="str">
-        <v>UPI/532184302317/AMRUTTULYA TEA/9766790749@paytm/HDFC BANK</v>
+        <v>UPI/363302703713/PUNE PRINTS/9714758754@paytm/HDFC BANK</v>
       </c>
       <c r="F27" t="str">
-        <v>152.00</v>
+        <v>164.00</v>
       </c>
       <c r="G27" t="str">
         <v>0.00</v>
       </c>
       <c r="H27" t="str">
-        <v>60446.12</v>
+        <v>60693.12</v>
       </c>
     </row>
     <row r="28">
@@ -996,25 +996,25 @@
         <v>22</v>
       </c>
       <c r="B28" t="str">
-        <v>10/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="C28" t="str">
-        <v>10/07/2026</v>
+        <v>12/07/2026</v>
       </c>
       <c r="D28" t="str">
         <v>-</v>
       </c>
       <c r="E28" t="str">
-        <v>UPI/529038106766/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
+        <v>ATM CASH WDL ATW 579760 PUNE FC ROAD</v>
       </c>
       <c r="F28" t="str">
-        <v>119.00</v>
+        <v>3000.00</v>
       </c>
       <c r="G28" t="str">
         <v>0.00</v>
       </c>
       <c r="H28" t="str">
-        <v>60327.12</v>
+        <v>57693.12</v>
       </c>
     </row>
     <row r="29">
@@ -1022,25 +1022,25 @@
         <v>23</v>
       </c>
       <c r="B29" t="str">
-        <v>10/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="C29" t="str">
-        <v>10/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="D29" t="str">
         <v>-</v>
       </c>
       <c r="E29" t="str">
-        <v>UPI/469221822172/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/902790179336/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
       </c>
       <c r="F29" t="str">
-        <v>698.00</v>
+        <v>299.00</v>
       </c>
       <c r="G29" t="str">
         <v>0.00</v>
       </c>
       <c r="H29" t="str">
-        <v>59629.12</v>
+        <v>57394.12</v>
       </c>
     </row>
     <row r="30">
@@ -1048,25 +1048,25 @@
         <v>24</v>
       </c>
       <c r="B30" t="str">
-        <v>11/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="C30" t="str">
-        <v>11/07/2026</v>
+        <v>13/07/2026</v>
       </c>
       <c r="D30" t="str">
         <v>-</v>
       </c>
       <c r="E30" t="str">
-        <v>UPI/482764614420/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/883075535087/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F30" t="str">
-        <v>377.00</v>
+        <v>299.00</v>
       </c>
       <c r="G30" t="str">
         <v>0.00</v>
       </c>
       <c r="H30" t="str">
-        <v>59252.12</v>
+        <v>57095.12</v>
       </c>
     </row>
     <row r="31">
@@ -1074,25 +1074,25 @@
         <v>25</v>
       </c>
       <c r="B31" t="str">
-        <v>11/07/2026</v>
+        <v>14/07/2026</v>
       </c>
       <c r="C31" t="str">
-        <v>11/07/2026</v>
+        <v>14/07/2026</v>
       </c>
       <c r="D31" t="str">
         <v>-</v>
       </c>
       <c r="E31" t="str">
-        <v>UPI/402802400197/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/807621439895/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F31" t="str">
-        <v>285.00</v>
+        <v>310.00</v>
       </c>
       <c r="G31" t="str">
         <v>0.00</v>
       </c>
       <c r="H31" t="str">
-        <v>58967.12</v>
+        <v>56785.12</v>
       </c>
     </row>
     <row r="32">
@@ -1100,25 +1100,25 @@
         <v>26</v>
       </c>
       <c r="B32" t="str">
-        <v>12/07/2026</v>
+        <v>14/07/2026</v>
       </c>
       <c r="C32" t="str">
-        <v>12/07/2026</v>
+        <v>14/07/2026</v>
       </c>
       <c r="D32" t="str">
         <v>-</v>
       </c>
       <c r="E32" t="str">
-        <v>ATM CASH WDL ATW 259171 PUNE FC ROAD</v>
+        <v>UPI/137863319320/GOODLUCK CAFE/9760954517@paytm/HDFC BANK</v>
       </c>
       <c r="F32" t="str">
-        <v>3000.00</v>
+        <v>194.00</v>
       </c>
       <c r="G32" t="str">
         <v>0.00</v>
       </c>
       <c r="H32" t="str">
-        <v>55967.12</v>
+        <v>56591.12</v>
       </c>
     </row>
     <row r="33">
@@ -1126,25 +1126,25 @@
         <v>27</v>
       </c>
       <c r="B33" t="str">
-        <v>13/07/2026</v>
+        <v>15/07/2026</v>
       </c>
       <c r="C33" t="str">
-        <v>13/07/2026</v>
+        <v>15/07/2026</v>
       </c>
       <c r="D33" t="str">
         <v>-</v>
       </c>
       <c r="E33" t="str">
-        <v>UPI/902790179336/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
+        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/498559698</v>
       </c>
       <c r="F33" t="str">
-        <v>299.00</v>
+        <v>4210.00</v>
       </c>
       <c r="G33" t="str">
         <v>0.00</v>
       </c>
       <c r="H33" t="str">
-        <v>55668.12</v>
+        <v>52381.12</v>
       </c>
     </row>
     <row r="34">
@@ -1152,25 +1152,25 @@
         <v>28</v>
       </c>
       <c r="B34" t="str">
-        <v>13/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="C34" t="str">
-        <v>13/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="D34" t="str">
         <v>-</v>
       </c>
       <c r="E34" t="str">
-        <v>UPI/883075535087/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
+        <v>UPI/840986514487/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F34" t="str">
-        <v>299.00</v>
+        <v>215.00</v>
       </c>
       <c r="G34" t="str">
         <v>0.00</v>
       </c>
       <c r="H34" t="str">
-        <v>55369.12</v>
+        <v>52166.12</v>
       </c>
     </row>
     <row r="35">
@@ -1178,25 +1178,25 @@
         <v>29</v>
       </c>
       <c r="B35" t="str">
-        <v>14/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="C35" t="str">
-        <v>14/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="D35" t="str">
         <v>-</v>
       </c>
       <c r="E35" t="str">
-        <v>UPI/441100894310/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/918376975366/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F35" t="str">
-        <v>268.00</v>
+        <v>363.00</v>
       </c>
       <c r="G35" t="str">
         <v>0.00</v>
       </c>
       <c r="H35" t="str">
-        <v>55101.12</v>
+        <v>51803.12</v>
       </c>
     </row>
     <row r="36">
@@ -1204,25 +1204,25 @@
         <v>30</v>
       </c>
       <c r="B36" t="str">
-        <v>15/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="C36" t="str">
-        <v>15/07/2026</v>
+        <v>16/07/2026</v>
       </c>
       <c r="D36" t="str">
         <v>-</v>
       </c>
       <c r="E36" t="str">
-        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/498559698</v>
+        <v>UPI/485184686328/GOODLUCK CAFE/9721891649@paytm/HDFC BANK</v>
       </c>
       <c r="F36" t="str">
-        <v>4210.00</v>
+        <v>44.00</v>
       </c>
       <c r="G36" t="str">
         <v>0.00</v>
       </c>
       <c r="H36" t="str">
-        <v>50891.12</v>
+        <v>51759.12</v>
       </c>
     </row>
     <row r="37">
@@ -1230,25 +1230,25 @@
         <v>31</v>
       </c>
       <c r="B37" t="str">
-        <v>15/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="C37" t="str">
-        <v>15/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="D37" t="str">
         <v>-</v>
       </c>
       <c r="E37" t="str">
-        <v>UPI/455796485324/VAISHALI CAFE/9730401978@paytm/HDFC BANK</v>
+        <v>UPI/798691390850/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
       </c>
       <c r="F37" t="str">
-        <v>60.00</v>
+        <v>1194.00</v>
       </c>
       <c r="G37" t="str">
         <v>0.00</v>
       </c>
       <c r="H37" t="str">
-        <v>50831.12</v>
+        <v>50565.12</v>
       </c>
     </row>
     <row r="38">
@@ -1256,25 +1256,25 @@
         <v>32</v>
       </c>
       <c r="B38" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="C38" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="D38" t="str">
         <v>-</v>
       </c>
       <c r="E38" t="str">
-        <v>UPI/539809515140/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/265162227768/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F38" t="str">
-        <v>301.00</v>
+        <v>350.00</v>
       </c>
       <c r="G38" t="str">
         <v>0.00</v>
       </c>
       <c r="H38" t="str">
-        <v>50530.12</v>
+        <v>50215.12</v>
       </c>
     </row>
     <row r="39">
@@ -1282,25 +1282,25 @@
         <v>33</v>
       </c>
       <c r="B39" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="C39" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="D39" t="str">
         <v>-</v>
       </c>
       <c r="E39" t="str">
-        <v>UPI/701921704551/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/339836605009/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F39" t="str">
-        <v>576.00</v>
+        <v>1469.00</v>
       </c>
       <c r="G39" t="str">
         <v>0.00</v>
       </c>
       <c r="H39" t="str">
-        <v>49954.12</v>
+        <v>48746.12</v>
       </c>
     </row>
     <row r="40">
@@ -1308,25 +1308,25 @@
         <v>34</v>
       </c>
       <c r="B40" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="C40" t="str">
-        <v>16/07/2026</v>
+        <v>17/07/2026</v>
       </c>
       <c r="D40" t="str">
         <v>-</v>
       </c>
       <c r="E40" t="str">
-        <v>UPI/601326226792/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/501330741168/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F40" t="str">
-        <v>626.00</v>
+        <v>241.00</v>
       </c>
       <c r="G40" t="str">
         <v>0.00</v>
       </c>
       <c r="H40" t="str">
-        <v>49328.12</v>
+        <v>48505.12</v>
       </c>
     </row>
     <row r="41">
@@ -1334,25 +1334,25 @@
         <v>35</v>
       </c>
       <c r="B41" t="str">
-        <v>16/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="C41" t="str">
-        <v>16/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="D41" t="str">
         <v>-</v>
       </c>
       <c r="E41" t="str">
-        <v>UPI/781128412159/AMRUTTULYA TEA/9711477683@paytm/HDFC BANK</v>
+        <v>UPI/919428245187/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F41" t="str">
-        <v>203.00</v>
+        <v>124.00</v>
       </c>
       <c r="G41" t="str">
         <v>0.00</v>
       </c>
       <c r="H41" t="str">
-        <v>49125.12</v>
+        <v>48381.12</v>
       </c>
     </row>
     <row r="42">
@@ -1360,25 +1360,25 @@
         <v>36</v>
       </c>
       <c r="B42" t="str">
-        <v>17/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="C42" t="str">
-        <v>17/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="D42" t="str">
         <v>-</v>
       </c>
       <c r="E42" t="str">
-        <v>UPI/798691390850/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
+        <v>UPI/825693140807/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F42" t="str">
-        <v>1194.00</v>
+        <v>271.00</v>
       </c>
       <c r="G42" t="str">
         <v>0.00</v>
       </c>
       <c r="H42" t="str">
-        <v>47931.12</v>
+        <v>48110.12</v>
       </c>
     </row>
     <row r="43">
@@ -1386,25 +1386,25 @@
         <v>37</v>
       </c>
       <c r="B43" t="str">
-        <v>17/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="C43" t="str">
-        <v>17/07/2026</v>
+        <v>18/07/2026</v>
       </c>
       <c r="D43" t="str">
         <v>-</v>
       </c>
       <c r="E43" t="str">
-        <v>UPI/277341241203/DMART/grocery@ybl/HDFC BANK</v>
+        <v>UPI/197180528845/PUNE PRINTS/9742577020@paytm/HDFC BANK</v>
       </c>
       <c r="F43" t="str">
-        <v>1012.00</v>
+        <v>96.00</v>
       </c>
       <c r="G43" t="str">
         <v>0.00</v>
       </c>
       <c r="H43" t="str">
-        <v>46919.12</v>
+        <v>48014.12</v>
       </c>
     </row>
     <row r="44">
@@ -1412,25 +1412,25 @@
         <v>38</v>
       </c>
       <c r="B44" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="C44" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="D44" t="str">
         <v>-</v>
       </c>
       <c r="E44" t="str">
-        <v>UPI/924452034616/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>NEFT-N201260478812-NORTHWIND MEDIA PVT LTD-INV 0715</v>
       </c>
       <c r="F44" t="str">
-        <v>289.00</v>
+        <v>0.00</v>
       </c>
       <c r="G44" t="str">
-        <v>0.00</v>
+        <v>42000.00</v>
       </c>
       <c r="H44" t="str">
-        <v>46630.12</v>
+        <v>90014.12</v>
       </c>
     </row>
     <row r="45">
@@ -1438,25 +1438,25 @@
         <v>39</v>
       </c>
       <c r="B45" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="C45" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="D45" t="str">
         <v>-</v>
       </c>
       <c r="E45" t="str">
-        <v>UPI/690093096368/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/824077950580/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F45" t="str">
-        <v>590.00</v>
+        <v>621.00</v>
       </c>
       <c r="G45" t="str">
         <v>0.00</v>
       </c>
       <c r="H45" t="str">
-        <v>46040.12</v>
+        <v>89393.12</v>
       </c>
     </row>
     <row r="46">
@@ -1464,25 +1464,25 @@
         <v>40</v>
       </c>
       <c r="B46" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="C46" t="str">
-        <v>18/07/2026</v>
+        <v>19/07/2026</v>
       </c>
       <c r="D46" t="str">
         <v>-</v>
       </c>
       <c r="E46" t="str">
-        <v>UPI/909748958982/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/849730837112/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F46" t="str">
-        <v>237.00</v>
+        <v>242.00</v>
       </c>
       <c r="G46" t="str">
         <v>0.00</v>
       </c>
       <c r="H46" t="str">
-        <v>45803.12</v>
+        <v>89151.12</v>
       </c>
     </row>
     <row r="47">
@@ -1490,25 +1490,25 @@
         <v>41</v>
       </c>
       <c r="B47" t="str">
-        <v>19/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="C47" t="str">
-        <v>19/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="D47" t="str">
         <v>-</v>
       </c>
       <c r="E47" t="str">
-        <v>NEFT-N201260478812-NORTHWIND MEDIA PVT LTD-INV 0715</v>
+        <v>UPI/406187161686/JIO PREPAID/jio@sbi/HDFC BANK</v>
       </c>
       <c r="F47" t="str">
-        <v>0.00</v>
+        <v>349.00</v>
       </c>
       <c r="G47" t="str">
-        <v>42000.00</v>
+        <v>0.00</v>
       </c>
       <c r="H47" t="str">
-        <v>87803.12</v>
+        <v>88802.12</v>
       </c>
     </row>
     <row r="48">
@@ -1516,25 +1516,25 @@
         <v>42</v>
       </c>
       <c r="B48" t="str">
-        <v>19/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="C48" t="str">
-        <v>19/07/2026</v>
+        <v>20/07/2026</v>
       </c>
       <c r="D48" t="str">
         <v>-</v>
       </c>
       <c r="E48" t="str">
-        <v>UPI/364175491803/PUNE PRINTS/9770139446@paytm/HDFC BANK</v>
+        <v>UPI/848686722293/VAISHALI CAFE/9742823109@paytm/HDFC BANK</v>
       </c>
       <c r="F48" t="str">
-        <v>175.00</v>
+        <v>150.00</v>
       </c>
       <c r="G48" t="str">
         <v>0.00</v>
       </c>
       <c r="H48" t="str">
-        <v>87628.12</v>
+        <v>88652.12</v>
       </c>
     </row>
     <row r="49">
@@ -1542,25 +1542,25 @@
         <v>43</v>
       </c>
       <c r="B49" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="C49" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="D49" t="str">
         <v>-</v>
       </c>
       <c r="E49" t="str">
-        <v>UPI/406187161686/JIO PREPAID/jio@sbi/HDFC BANK</v>
+        <v>UPI/452856088965/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F49" t="str">
-        <v>349.00</v>
+        <v>567.00</v>
       </c>
       <c r="G49" t="str">
         <v>0.00</v>
       </c>
       <c r="H49" t="str">
-        <v>87279.12</v>
+        <v>88085.12</v>
       </c>
     </row>
     <row r="50">
@@ -1568,25 +1568,25 @@
         <v>44</v>
       </c>
       <c r="B50" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="C50" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="D50" t="str">
         <v>-</v>
       </c>
       <c r="E50" t="str">
-        <v>UPI/942167452885/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/469753230852/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F50" t="str">
-        <v>412.00</v>
+        <v>342.00</v>
       </c>
       <c r="G50" t="str">
         <v>0.00</v>
       </c>
       <c r="H50" t="str">
-        <v>86867.12</v>
+        <v>87743.12</v>
       </c>
     </row>
     <row r="51">
@@ -1594,25 +1594,25 @@
         <v>45</v>
       </c>
       <c r="B51" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="C51" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="D51" t="str">
         <v>-</v>
       </c>
       <c r="E51" t="str">
-        <v>UPI/559871446574/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/402802400197/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F51" t="str">
-        <v>597.00</v>
+        <v>285.00</v>
       </c>
       <c r="G51" t="str">
         <v>0.00</v>
       </c>
       <c r="H51" t="str">
-        <v>86270.12</v>
+        <v>87458.12</v>
       </c>
     </row>
     <row r="52">
@@ -1620,25 +1620,25 @@
         <v>46</v>
       </c>
       <c r="B52" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="C52" t="str">
-        <v>20/07/2026</v>
+        <v>21/07/2026</v>
       </c>
       <c r="D52" t="str">
         <v>-</v>
       </c>
       <c r="E52" t="str">
-        <v>UPI/550214739539/VAISHALI CAFE/9776063776@paytm/HDFC BANK</v>
+        <v>UPI/466649379418/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F52" t="str">
-        <v>220.00</v>
+        <v>313.00</v>
       </c>
       <c r="G52" t="str">
         <v>0.00</v>
       </c>
       <c r="H52" t="str">
-        <v>86050.12</v>
+        <v>87145.12</v>
       </c>
     </row>
     <row r="53">
@@ -1655,16 +1655,16 @@
         <v>-</v>
       </c>
       <c r="E53" t="str">
-        <v>UPI/466581942187/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/966429442213/AMRUTTULYA TEA/9740731326@paytm/HDFC BANK</v>
       </c>
       <c r="F53" t="str">
-        <v>370.00</v>
+        <v>89.00</v>
       </c>
       <c r="G53" t="str">
         <v>0.00</v>
       </c>
       <c r="H53" t="str">
-        <v>85680.12</v>
+        <v>87056.12</v>
       </c>
     </row>
     <row r="54">
@@ -1681,16 +1681,16 @@
         <v>-</v>
       </c>
       <c r="E54" t="str">
-        <v>UPI/658707792731/GOODLUCK CAFE/9719704438@paytm/HDFC BANK</v>
+        <v>UPI/345714846695/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F54" t="str">
-        <v>208.00</v>
+        <v>656.00</v>
       </c>
       <c r="G54" t="str">
         <v>0.00</v>
       </c>
       <c r="H54" t="str">
-        <v>85472.12</v>
+        <v>86400.12</v>
       </c>
     </row>
     <row r="55">
@@ -1698,25 +1698,25 @@
         <v>49</v>
       </c>
       <c r="B55" t="str">
-        <v>23/07/2026</v>
+        <v>22/07/2026</v>
       </c>
       <c r="C55" t="str">
-        <v>23/07/2026</v>
+        <v>22/07/2026</v>
       </c>
       <c r="D55" t="str">
         <v>-</v>
       </c>
       <c r="E55" t="str">
-        <v>UPI/384624717035/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/340235174773/AMRUTTULYA TEA/9780399465@paytm/HDFC BANK</v>
       </c>
       <c r="F55" t="str">
-        <v>298.00</v>
+        <v>101.00</v>
       </c>
       <c r="G55" t="str">
         <v>0.00</v>
       </c>
       <c r="H55" t="str">
-        <v>85174.12</v>
+        <v>86299.12</v>
       </c>
     </row>
     <row r="56">
@@ -1733,16 +1733,16 @@
         <v>-</v>
       </c>
       <c r="E56" t="str">
-        <v>UPI/688856796664/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/619539803150/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F56" t="str">
-        <v>721.00</v>
+        <v>639.00</v>
       </c>
       <c r="G56" t="str">
         <v>0.00</v>
       </c>
       <c r="H56" t="str">
-        <v>84453.12</v>
+        <v>85660.12</v>
       </c>
     </row>
     <row r="57">
@@ -1759,16 +1759,16 @@
         <v>-</v>
       </c>
       <c r="E57" t="str">
-        <v>UPI/793987945606/GOODLUCK CAFE/9760135658@paytm/HDFC BANK</v>
+        <v>UPI/862223808141/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F57" t="str">
-        <v>191.00</v>
+        <v>982.00</v>
       </c>
       <c r="G57" t="str">
         <v>0.00</v>
       </c>
       <c r="H57" t="str">
-        <v>84262.12</v>
+        <v>84678.12</v>
       </c>
     </row>
     <row r="58">
@@ -1776,25 +1776,25 @@
         <v>52</v>
       </c>
       <c r="B58" t="str">
-        <v>25/07/2026</v>
+        <v>24/07/2026</v>
       </c>
       <c r="C58" t="str">
-        <v>25/07/2026</v>
+        <v>24/07/2026</v>
       </c>
       <c r="D58" t="str">
         <v>-</v>
       </c>
       <c r="E58" t="str">
-        <v>UPI/624578097253/AMRUTTULYA TEA/9721549089@paytm/HDFC BANK</v>
+        <v>UPI/469221822172/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F58" t="str">
-        <v>175.00</v>
+        <v>135.00</v>
       </c>
       <c r="G58" t="str">
         <v>0.00</v>
       </c>
       <c r="H58" t="str">
-        <v>84087.12</v>
+        <v>84543.12</v>
       </c>
     </row>
     <row r="59">
@@ -1802,25 +1802,25 @@
         <v>53</v>
       </c>
       <c r="B59" t="str">
-        <v>26/07/2026</v>
+        <v>25/07/2026</v>
       </c>
       <c r="C59" t="str">
-        <v>26/07/2026</v>
+        <v>25/07/2026</v>
       </c>
       <c r="D59" t="str">
         <v>-</v>
       </c>
       <c r="E59" t="str">
-        <v>UPI/265162227768/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/929309284221/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F59" t="str">
-        <v>350.00</v>
+        <v>572.00</v>
       </c>
       <c r="G59" t="str">
         <v>0.00</v>
       </c>
       <c r="H59" t="str">
-        <v>83737.12</v>
+        <v>83971.12</v>
       </c>
     </row>
     <row r="60">
@@ -1837,16 +1837,16 @@
         <v>-</v>
       </c>
       <c r="E60" t="str">
-        <v>UPI/382968674250/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/623731127940/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F60" t="str">
-        <v>605.00</v>
+        <v>552.00</v>
       </c>
       <c r="G60" t="str">
         <v>0.00</v>
       </c>
       <c r="H60" t="str">
-        <v>83132.12</v>
+        <v>83419.12</v>
       </c>
     </row>
     <row r="61">
@@ -1863,16 +1863,16 @@
         <v>-</v>
       </c>
       <c r="E61" t="str">
-        <v>UPI/214986923872/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/973984938138/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F61" t="str">
-        <v>416.00</v>
+        <v>313.00</v>
       </c>
       <c r="G61" t="str">
         <v>0.00</v>
       </c>
       <c r="H61" t="str">
-        <v>82716.12</v>
+        <v>83106.12</v>
       </c>
     </row>
     <row r="62">
@@ -1889,16 +1889,16 @@
         <v>-</v>
       </c>
       <c r="E62" t="str">
-        <v>UPI/466649379418/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/575572560238/AMRUTTULYA TEA/9744885580@paytm/HDFC BANK</v>
       </c>
       <c r="F62" t="str">
-        <v>546.00</v>
+        <v>91.00</v>
       </c>
       <c r="G62" t="str">
         <v>0.00</v>
       </c>
       <c r="H62" t="str">
-        <v>82170.12</v>
+        <v>83015.12</v>
       </c>
     </row>
     <row r="63">
@@ -1915,16 +1915,16 @@
         <v>-</v>
       </c>
       <c r="E63" t="str">
-        <v>UPI/168306790827/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/379442413244/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F63" t="str">
-        <v>391.00</v>
+        <v>196.00</v>
       </c>
       <c r="G63" t="str">
         <v>0.00</v>
       </c>
       <c r="H63" t="str">
-        <v>81779.12</v>
+        <v>82819.12</v>
       </c>
     </row>
     <row r="64">
@@ -1941,7 +1941,7 @@
         <v>-</v>
       </c>
       <c r="E64" t="str">
-        <v>UPI/945014500198/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
+        <v>UPI/796468232269/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
       </c>
       <c r="F64" t="str">
         <v>1999.00</v>
@@ -1950,7 +1950,7 @@
         <v>0.00</v>
       </c>
       <c r="H64" t="str">
-        <v>79780.12</v>
+        <v>80820.12</v>
       </c>
     </row>
     <row r="65">
@@ -1958,25 +1958,25 @@
         <v>59</v>
       </c>
       <c r="B65" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="C65" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="D65" t="str">
         <v>-</v>
       </c>
       <c r="E65" t="str">
-        <v>UPI/232459618570/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
+        <v>UPI/987109972559/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F65" t="str">
-        <v>1675.28</v>
+        <v>459.00</v>
       </c>
       <c r="G65" t="str">
         <v>0.00</v>
       </c>
       <c r="H65" t="str">
-        <v>78104.84</v>
+        <v>80361.12</v>
       </c>
     </row>
     <row r="66">
@@ -1984,25 +1984,25 @@
         <v>60</v>
       </c>
       <c r="B66" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="C66" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="D66" t="str">
         <v>-</v>
       </c>
       <c r="E66" t="str">
-        <v>UPI/516034200694/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/565825937176/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F66" t="str">
-        <v>254.00</v>
+        <v>149.00</v>
       </c>
       <c r="G66" t="str">
         <v>0.00</v>
       </c>
       <c r="H66" t="str">
-        <v>77850.84</v>
+        <v>80212.12</v>
       </c>
     </row>
     <row r="67">
@@ -2010,25 +2010,25 @@
         <v>61</v>
       </c>
       <c r="B67" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="C67" t="str">
-        <v>03/08/2026</v>
+        <v>02/08/2026</v>
       </c>
       <c r="D67" t="str">
         <v>-</v>
       </c>
       <c r="E67" t="str">
-        <v>UPI/517858404992/DMART/grocery@ybl/HDFC BANK</v>
+        <v>UPI/517858404992/VAISHALI CAFE/9709298667@paytm/HDFC BANK</v>
       </c>
       <c r="F67" t="str">
-        <v>1540.00</v>
+        <v>141.00</v>
       </c>
       <c r="G67" t="str">
         <v>0.00</v>
       </c>
       <c r="H67" t="str">
-        <v>76310.84</v>
+        <v>80071.12</v>
       </c>
     </row>
     <row r="68">
@@ -2045,16 +2045,16 @@
         <v>-</v>
       </c>
       <c r="E68" t="str">
-        <v>UPI/941377109615/PUNE PRINTS/9717573173@paytm/HDFC BANK</v>
+        <v>UPI/893694590427/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F68" t="str">
-        <v>168.00</v>
+        <v>1675.28</v>
       </c>
       <c r="G68" t="str">
         <v>0.00</v>
       </c>
       <c r="H68" t="str">
-        <v>76142.84</v>
+        <v>78395.84</v>
       </c>
     </row>
     <row r="69">
@@ -2062,25 +2062,25 @@
         <v>63</v>
       </c>
       <c r="B69" t="str">
-        <v>04/08/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="C69" t="str">
-        <v>04/08/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="D69" t="str">
         <v>-</v>
       </c>
       <c r="E69" t="str">
-        <v>UPI/820397937390/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/558755666692/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F69" t="str">
-        <v>510.00</v>
+        <v>374.00</v>
       </c>
       <c r="G69" t="str">
         <v>0.00</v>
       </c>
       <c r="H69" t="str">
-        <v>75632.84</v>
+        <v>78021.84</v>
       </c>
     </row>
     <row r="70">
@@ -2088,25 +2088,25 @@
         <v>64</v>
       </c>
       <c r="B70" t="str">
-        <v>04/08/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="C70" t="str">
-        <v>04/08/2026</v>
+        <v>03/08/2026</v>
       </c>
       <c r="D70" t="str">
         <v>-</v>
       </c>
       <c r="E70" t="str">
-        <v>UPI/987109972559/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/333094548480/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F70" t="str">
-        <v>459.00</v>
+        <v>1931.00</v>
       </c>
       <c r="G70" t="str">
         <v>0.00</v>
       </c>
       <c r="H70" t="str">
-        <v>75173.84</v>
+        <v>76090.84</v>
       </c>
     </row>
     <row r="71">
@@ -2114,25 +2114,25 @@
         <v>65</v>
       </c>
       <c r="B71" t="str">
-        <v>05/08/2026</v>
+        <v>04/08/2026</v>
       </c>
       <c r="C71" t="str">
-        <v>05/08/2026</v>
+        <v>04/08/2026</v>
       </c>
       <c r="D71" t="str">
         <v>-</v>
       </c>
       <c r="E71" t="str">
-        <v>MMT/IMPS/210703252512/Rent Aug/Meera Kulkarni/HDFC0001234</v>
+        <v>UPI/854979805112/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F71" t="str">
-        <v>18500.00</v>
+        <v>354.00</v>
       </c>
       <c r="G71" t="str">
         <v>0.00</v>
       </c>
       <c r="H71" t="str">
-        <v>56673.84</v>
+        <v>75736.84</v>
       </c>
     </row>
     <row r="72">
@@ -2140,25 +2140,25 @@
         <v>66</v>
       </c>
       <c r="B72" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="C72" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="D72" t="str">
         <v>-</v>
       </c>
       <c r="E72" t="str">
-        <v>UPI/657795200031/NOTION LABS/notion@icici/HDFC BANK</v>
+        <v>MMT/IMPS/364175491803/Rent Aug/Meera Kulkarni/HDFC0001234</v>
       </c>
       <c r="F72" t="str">
-        <v>880.00</v>
+        <v>18500.00</v>
       </c>
       <c r="G72" t="str">
         <v>0.00</v>
       </c>
       <c r="H72" t="str">
-        <v>55793.84</v>
+        <v>57236.84</v>
       </c>
     </row>
     <row r="73">
@@ -2166,25 +2166,25 @@
         <v>67</v>
       </c>
       <c r="B73" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="C73" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="D73" t="str">
         <v>-</v>
       </c>
       <c r="E73" t="str">
-        <v>UPI/435785861825/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/945014500198/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F73" t="str">
-        <v>228.00</v>
+        <v>261.00</v>
       </c>
       <c r="G73" t="str">
         <v>0.00</v>
       </c>
       <c r="H73" t="str">
-        <v>55565.84</v>
+        <v>56975.84</v>
       </c>
     </row>
     <row r="74">
@@ -2192,25 +2192,25 @@
         <v>68</v>
       </c>
       <c r="B74" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="C74" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="D74" t="str">
         <v>-</v>
       </c>
       <c r="E74" t="str">
-        <v>UPI/879231223813/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/292604105593/AMRUTTULYA TEA/9765913720@paytm/HDFC BANK</v>
       </c>
       <c r="F74" t="str">
-        <v>165.00</v>
+        <v>88.00</v>
       </c>
       <c r="G74" t="str">
         <v>0.00</v>
       </c>
       <c r="H74" t="str">
-        <v>55400.84</v>
+        <v>56887.84</v>
       </c>
     </row>
     <row r="75">
@@ -2218,25 +2218,25 @@
         <v>69</v>
       </c>
       <c r="B75" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="C75" t="str">
-        <v>06/08/2026</v>
+        <v>05/08/2026</v>
       </c>
       <c r="D75" t="str">
         <v>-</v>
       </c>
       <c r="E75" t="str">
-        <v>UPI/540286793489/AMRUTTULYA TEA/9732525227@paytm/HDFC BANK</v>
+        <v>UPI/543009731429/PUNE PRINTS/9784351783@paytm/HDFC BANK</v>
       </c>
       <c r="F75" t="str">
-        <v>138.00</v>
+        <v>135.00</v>
       </c>
       <c r="G75" t="str">
         <v>0.00</v>
       </c>
       <c r="H75" t="str">
-        <v>55262.84</v>
+        <v>56752.84</v>
       </c>
     </row>
     <row r="76">
@@ -2253,16 +2253,16 @@
         <v>-</v>
       </c>
       <c r="E76" t="str">
-        <v>UPI/277049520169/GOODLUCK CAFE/9733092464@paytm/HDFC BANK</v>
+        <v>UPI/293941807677/NOTION LABS/notion@icici/HDFC BANK</v>
       </c>
       <c r="F76" t="str">
-        <v>44.00</v>
+        <v>880.00</v>
       </c>
       <c r="G76" t="str">
         <v>0.00</v>
       </c>
       <c r="H76" t="str">
-        <v>55218.84</v>
+        <v>55872.84</v>
       </c>
     </row>
     <row r="77">
@@ -2270,25 +2270,25 @@
         <v>71</v>
       </c>
       <c r="B77" t="str">
-        <v>07/08/2026</v>
+        <v>08/08/2026</v>
       </c>
       <c r="C77" t="str">
-        <v>07/08/2026</v>
+        <v>08/08/2026</v>
       </c>
       <c r="D77" t="str">
         <v>-</v>
       </c>
       <c r="E77" t="str">
-        <v>UPI/337549306219/VAISHALI CAFE/9783719500@paytm/HDFC BANK</v>
+        <v>UPI/624578097253/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
       </c>
       <c r="F77" t="str">
-        <v>105.00</v>
+        <v>1567.00</v>
       </c>
       <c r="G77" t="str">
         <v>0.00</v>
       </c>
       <c r="H77" t="str">
-        <v>55113.84</v>
+        <v>54305.84</v>
       </c>
     </row>
     <row r="78">
@@ -2296,25 +2296,25 @@
         <v>72</v>
       </c>
       <c r="B78" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="C78" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="D78" t="str">
         <v>-</v>
       </c>
       <c r="E78" t="str">
-        <v>UPI/610382137238/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
+        <v>UPI/207364072650/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F78" t="str">
-        <v>1567.00</v>
+        <v>638.00</v>
       </c>
       <c r="G78" t="str">
         <v>0.00</v>
       </c>
       <c r="H78" t="str">
-        <v>53546.84</v>
+        <v>53667.84</v>
       </c>
     </row>
     <row r="79">
@@ -2322,25 +2322,25 @@
         <v>73</v>
       </c>
       <c r="B79" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="C79" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="D79" t="str">
         <v>-</v>
       </c>
       <c r="E79" t="str">
-        <v>UPI/643832732387/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>ECS RETURN CHG BAJAJ FINANCE INSUFF BAL</v>
       </c>
       <c r="F79" t="str">
-        <v>287.00</v>
+        <v>590.00</v>
       </c>
       <c r="G79" t="str">
         <v>0.00</v>
       </c>
       <c r="H79" t="str">
-        <v>53259.84</v>
+        <v>53077.84</v>
       </c>
     </row>
     <row r="80">
@@ -2348,25 +2348,25 @@
         <v>74</v>
       </c>
       <c r="B80" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="C80" t="str">
-        <v>08/08/2026</v>
+        <v>09/08/2026</v>
       </c>
       <c r="D80" t="str">
         <v>-</v>
       </c>
       <c r="E80" t="str">
-        <v>UPI/824656565720/VAISHALI CAFE/9790477313@paytm/HDFC BANK</v>
+        <v>GST ON ECS RETURN CHG</v>
       </c>
       <c r="F80" t="str">
-        <v>211.00</v>
+        <v>106.20</v>
       </c>
       <c r="G80" t="str">
         <v>0.00</v>
       </c>
       <c r="H80" t="str">
-        <v>53048.84</v>
+        <v>52971.64</v>
       </c>
     </row>
     <row r="81">
@@ -2374,25 +2374,25 @@
         <v>75</v>
       </c>
       <c r="B81" t="str">
-        <v>09/08/2026</v>
+        <v>10/08/2026</v>
       </c>
       <c r="C81" t="str">
-        <v>09/08/2026</v>
+        <v>10/08/2026</v>
       </c>
       <c r="D81" t="str">
         <v>-</v>
       </c>
       <c r="E81" t="str">
-        <v>UPI/800245331157/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/754175627604/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
       </c>
       <c r="F81" t="str">
-        <v>239.00</v>
+        <v>119.00</v>
       </c>
       <c r="G81" t="str">
         <v>0.00</v>
       </c>
       <c r="H81" t="str">
-        <v>52809.84</v>
+        <v>52852.64</v>
       </c>
     </row>
     <row r="82">
@@ -2400,25 +2400,25 @@
         <v>76</v>
       </c>
       <c r="B82" t="str">
-        <v>09/08/2026</v>
+        <v>10/08/2026</v>
       </c>
       <c r="C82" t="str">
-        <v>09/08/2026</v>
+        <v>10/08/2026</v>
       </c>
       <c r="D82" t="str">
         <v>-</v>
       </c>
       <c r="E82" t="str">
-        <v>ECS RETURN CHG BAJAJ FINANCE INSUFF BAL</v>
+        <v>UPI/216005764529/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F82" t="str">
-        <v>590.00</v>
+        <v>1614.00</v>
       </c>
       <c r="G82" t="str">
         <v>0.00</v>
       </c>
       <c r="H82" t="str">
-        <v>52219.84</v>
+        <v>51238.64</v>
       </c>
     </row>
     <row r="83">
@@ -2426,25 +2426,25 @@
         <v>77</v>
       </c>
       <c r="B83" t="str">
-        <v>09/08/2026</v>
+        <v>11/08/2026</v>
       </c>
       <c r="C83" t="str">
-        <v>09/08/2026</v>
+        <v>11/08/2026</v>
       </c>
       <c r="D83" t="str">
         <v>-</v>
       </c>
       <c r="E83" t="str">
-        <v>GST ON ECS RETURN CHG</v>
+        <v>UPI/171804632782/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F83" t="str">
-        <v>106.20</v>
+        <v>244.00</v>
       </c>
       <c r="G83" t="str">
         <v>0.00</v>
       </c>
       <c r="H83" t="str">
-        <v>52113.64</v>
+        <v>50994.64</v>
       </c>
     </row>
     <row r="84">
@@ -2452,25 +2452,25 @@
         <v>78</v>
       </c>
       <c r="B84" t="str">
-        <v>10/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="C84" t="str">
-        <v>10/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="D84" t="str">
         <v>-</v>
       </c>
       <c r="E84" t="str">
-        <v>UPI/857252340018/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
+        <v>UPI/275382041954/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F84" t="str">
-        <v>119.00</v>
+        <v>435.00</v>
       </c>
       <c r="G84" t="str">
         <v>0.00</v>
       </c>
       <c r="H84" t="str">
-        <v>51994.64</v>
+        <v>50559.64</v>
       </c>
     </row>
     <row r="85">
@@ -2478,25 +2478,25 @@
         <v>79</v>
       </c>
       <c r="B85" t="str">
-        <v>10/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="C85" t="str">
-        <v>10/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="D85" t="str">
         <v>-</v>
       </c>
       <c r="E85" t="str">
-        <v>UPI/757677655690/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/102303143311/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F85" t="str">
-        <v>874.00</v>
+        <v>152.00</v>
       </c>
       <c r="G85" t="str">
         <v>0.00</v>
       </c>
       <c r="H85" t="str">
-        <v>51120.64</v>
+        <v>50407.64</v>
       </c>
     </row>
     <row r="86">
@@ -2504,25 +2504,25 @@
         <v>80</v>
       </c>
       <c r="B86" t="str">
-        <v>11/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="C86" t="str">
-        <v>11/08/2026</v>
+        <v>12/08/2026</v>
       </c>
       <c r="D86" t="str">
         <v>-</v>
       </c>
       <c r="E86" t="str">
-        <v>UPI/797660261904/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/643832732387/GOODLUCK CAFE/9725741012@paytm/HDFC BANK</v>
       </c>
       <c r="F86" t="str">
-        <v>281.00</v>
+        <v>159.00</v>
       </c>
       <c r="G86" t="str">
         <v>0.00</v>
       </c>
       <c r="H86" t="str">
-        <v>50839.64</v>
+        <v>50248.64</v>
       </c>
     </row>
     <row r="87">
@@ -2539,16 +2539,16 @@
         <v>-</v>
       </c>
       <c r="E87" t="str">
-        <v>UPI/210715855751/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>ATM CASH WDL ATW 171505 PUNE FC ROAD</v>
       </c>
       <c r="F87" t="str">
-        <v>213.00</v>
+        <v>3000.00</v>
       </c>
       <c r="G87" t="str">
         <v>0.00</v>
       </c>
       <c r="H87" t="str">
-        <v>50626.64</v>
+        <v>47248.64</v>
       </c>
     </row>
     <row r="88">
@@ -2556,25 +2556,25 @@
         <v>82</v>
       </c>
       <c r="B88" t="str">
-        <v>12/08/2026</v>
+        <v>13/08/2026</v>
       </c>
       <c r="C88" t="str">
-        <v>12/08/2026</v>
+        <v>13/08/2026</v>
       </c>
       <c r="D88" t="str">
         <v>-</v>
       </c>
       <c r="E88" t="str">
-        <v>UPI/132672077068/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/692722915555/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
       </c>
       <c r="F88" t="str">
-        <v>235.00</v>
+        <v>299.00</v>
       </c>
       <c r="G88" t="str">
         <v>0.00</v>
       </c>
       <c r="H88" t="str">
-        <v>50391.64</v>
+        <v>46949.64</v>
       </c>
     </row>
     <row r="89">
@@ -2582,25 +2582,25 @@
         <v>83</v>
       </c>
       <c r="B89" t="str">
-        <v>12/08/2026</v>
+        <v>13/08/2026</v>
       </c>
       <c r="C89" t="str">
-        <v>12/08/2026</v>
+        <v>13/08/2026</v>
       </c>
       <c r="D89" t="str">
         <v>-</v>
       </c>
       <c r="E89" t="str">
-        <v>ATM CASH WDL ATW 786140 PUNE FC ROAD</v>
+        <v>UPI/731255020434/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F89" t="str">
-        <v>3000.00</v>
+        <v>299.00</v>
       </c>
       <c r="G89" t="str">
         <v>0.00</v>
       </c>
       <c r="H89" t="str">
-        <v>47391.64</v>
+        <v>46650.64</v>
       </c>
     </row>
     <row r="90">
@@ -2617,16 +2617,16 @@
         <v>-</v>
       </c>
       <c r="E90" t="str">
-        <v>UPI/611932405433/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
+        <v>UPI/466766104334/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F90" t="str">
-        <v>299.00</v>
+        <v>300.00</v>
       </c>
       <c r="G90" t="str">
         <v>0.00</v>
       </c>
       <c r="H90" t="str">
-        <v>47092.64</v>
+        <v>46350.64</v>
       </c>
     </row>
     <row r="91">
@@ -2643,16 +2643,16 @@
         <v>-</v>
       </c>
       <c r="E91" t="str">
-        <v>UPI/617526690452/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
+        <v>UPI/785480889095/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F91" t="str">
-        <v>299.00</v>
+        <v>482.00</v>
       </c>
       <c r="G91" t="str">
         <v>0.00</v>
       </c>
       <c r="H91" t="str">
-        <v>46793.64</v>
+        <v>45868.64</v>
       </c>
     </row>
     <row r="92">
@@ -2660,25 +2660,25 @@
         <v>86</v>
       </c>
       <c r="B92" t="str">
-        <v>13/08/2026</v>
+        <v>14/08/2026</v>
       </c>
       <c r="C92" t="str">
-        <v>13/08/2026</v>
+        <v>14/08/2026</v>
       </c>
       <c r="D92" t="str">
         <v>-</v>
       </c>
       <c r="E92" t="str">
-        <v>UPI/828855094965/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/454861766076/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F92" t="str">
-        <v>490.00</v>
+        <v>339.00</v>
       </c>
       <c r="G92" t="str">
         <v>0.00</v>
       </c>
       <c r="H92" t="str">
-        <v>46303.64</v>
+        <v>45529.64</v>
       </c>
     </row>
     <row r="93">
@@ -2695,16 +2695,16 @@
         <v>-</v>
       </c>
       <c r="E93" t="str">
-        <v>UPI/573323830985/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/288003455172/GOODLUCK CAFE/9742821787@paytm/HDFC BANK</v>
       </c>
       <c r="F93" t="str">
-        <v>231.00</v>
+        <v>99.00</v>
       </c>
       <c r="G93" t="str">
         <v>0.00</v>
       </c>
       <c r="H93" t="str">
-        <v>46072.64</v>
+        <v>45430.64</v>
       </c>
     </row>
     <row r="94">
@@ -2721,7 +2721,7 @@
         <v>-</v>
       </c>
       <c r="E94" t="str">
-        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/854979805</v>
+        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/753155990</v>
       </c>
       <c r="F94" t="str">
         <v>4210.00</v>
@@ -2730,7 +2730,7 @@
         <v>0.00</v>
       </c>
       <c r="H94" t="str">
-        <v>41862.64</v>
+        <v>41220.64</v>
       </c>
     </row>
     <row r="95">
@@ -2747,16 +2747,16 @@
         <v>-</v>
       </c>
       <c r="E95" t="str">
-        <v>UPI/732779892510/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/993542517675/PUNE PRINTS/9716516997@paytm/HDFC BANK</v>
       </c>
       <c r="F95" t="str">
-        <v>522.00</v>
+        <v>151.00</v>
       </c>
       <c r="G95" t="str">
         <v>0.00</v>
       </c>
       <c r="H95" t="str">
-        <v>41340.64</v>
+        <v>41069.64</v>
       </c>
     </row>
     <row r="96">
@@ -2764,25 +2764,25 @@
         <v>90</v>
       </c>
       <c r="B96" t="str">
-        <v>15/08/2026</v>
+        <v>16/08/2026</v>
       </c>
       <c r="C96" t="str">
-        <v>15/08/2026</v>
+        <v>16/08/2026</v>
       </c>
       <c r="D96" t="str">
         <v>-</v>
       </c>
       <c r="E96" t="str">
-        <v>UPI/602417996292/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/203299151989/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F96" t="str">
-        <v>436.00</v>
+        <v>553.00</v>
       </c>
       <c r="G96" t="str">
         <v>0.00</v>
       </c>
       <c r="H96" t="str">
-        <v>40904.64</v>
+        <v>40516.64</v>
       </c>
     </row>
     <row r="97">
@@ -2790,25 +2790,25 @@
         <v>91</v>
       </c>
       <c r="B97" t="str">
-        <v>15/08/2026</v>
+        <v>16/08/2026</v>
       </c>
       <c r="C97" t="str">
-        <v>15/08/2026</v>
+        <v>16/08/2026</v>
       </c>
       <c r="D97" t="str">
         <v>-</v>
       </c>
       <c r="E97" t="str">
-        <v>UPI/646642764378/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/857252340018/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F97" t="str">
-        <v>425.00</v>
+        <v>463.00</v>
       </c>
       <c r="G97" t="str">
         <v>0.00</v>
       </c>
       <c r="H97" t="str">
-        <v>40479.64</v>
+        <v>40053.64</v>
       </c>
     </row>
     <row r="98">
@@ -2825,16 +2825,16 @@
         <v>-</v>
       </c>
       <c r="E98" t="str">
-        <v>UPI/916084683267/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/682115609128/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F98" t="str">
-        <v>487.00</v>
+        <v>255.00</v>
       </c>
       <c r="G98" t="str">
         <v>0.00</v>
       </c>
       <c r="H98" t="str">
-        <v>39992.64</v>
+        <v>39798.64</v>
       </c>
     </row>
     <row r="99">
@@ -2842,25 +2842,25 @@
         <v>93</v>
       </c>
       <c r="B99" t="str">
-        <v>16/08/2026</v>
+        <v>17/08/2026</v>
       </c>
       <c r="C99" t="str">
-        <v>16/08/2026</v>
+        <v>17/08/2026</v>
       </c>
       <c r="D99" t="str">
         <v>-</v>
       </c>
       <c r="E99" t="str">
-        <v>UPI/216005764529/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/792438158742/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
       </c>
       <c r="F99" t="str">
-        <v>476.00</v>
+        <v>1199.00</v>
       </c>
       <c r="G99" t="str">
         <v>0.00</v>
       </c>
       <c r="H99" t="str">
-        <v>39516.64</v>
+        <v>38599.64</v>
       </c>
     </row>
     <row r="100">
@@ -2877,16 +2877,16 @@
         <v>-</v>
       </c>
       <c r="E100" t="str">
-        <v>UPI/406715882290/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
+        <v>UPI/924176736874/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F100" t="str">
-        <v>1358.00</v>
+        <v>1268.00</v>
       </c>
       <c r="G100" t="str">
         <v>0.00</v>
       </c>
       <c r="H100" t="str">
-        <v>38158.64</v>
+        <v>37331.64</v>
       </c>
     </row>
     <row r="101">
@@ -2894,25 +2894,25 @@
         <v>95</v>
       </c>
       <c r="B101" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="C101" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="D101" t="str">
         <v>-</v>
       </c>
       <c r="E101" t="str">
-        <v>UPI/454861766076/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/249172279168/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F101" t="str">
-        <v>339.00</v>
+        <v>411.00</v>
       </c>
       <c r="G101" t="str">
         <v>0.00</v>
       </c>
       <c r="H101" t="str">
-        <v>37819.64</v>
+        <v>36920.64</v>
       </c>
     </row>
     <row r="102">
@@ -2920,25 +2920,25 @@
         <v>96</v>
       </c>
       <c r="B102" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="C102" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="D102" t="str">
         <v>-</v>
       </c>
       <c r="E102" t="str">
-        <v>UPI/364485755702/DMART/grocery@ybl/HDFC BANK</v>
+        <v>UPI/610925622144/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F102" t="str">
-        <v>1284.00</v>
+        <v>305.00</v>
       </c>
       <c r="G102" t="str">
         <v>0.00</v>
       </c>
       <c r="H102" t="str">
-        <v>36535.64</v>
+        <v>36615.64</v>
       </c>
     </row>
     <row r="103">
@@ -2946,25 +2946,25 @@
         <v>97</v>
       </c>
       <c r="B103" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="C103" t="str">
-        <v>17/08/2026</v>
+        <v>18/08/2026</v>
       </c>
       <c r="D103" t="str">
         <v>-</v>
       </c>
       <c r="E103" t="str">
-        <v>UPI/964258882589/VAISHALI CAFE/9717450104@paytm/HDFC BANK</v>
+        <v>UPI/717995059583/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F103" t="str">
-        <v>202.00</v>
+        <v>235.00</v>
       </c>
       <c r="G103" t="str">
         <v>0.00</v>
       </c>
       <c r="H103" t="str">
-        <v>36333.64</v>
+        <v>36380.64</v>
       </c>
     </row>
     <row r="104">
@@ -2972,25 +2972,25 @@
         <v>98</v>
       </c>
       <c r="B104" t="str">
-        <v>18/08/2026</v>
+        <v>19/08/2026</v>
       </c>
       <c r="C104" t="str">
-        <v>18/08/2026</v>
+        <v>19/08/2026</v>
       </c>
       <c r="D104" t="str">
         <v>-</v>
       </c>
       <c r="E104" t="str">
-        <v>UPI/801109818019/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/388694588048/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F104" t="str">
-        <v>393.00</v>
+        <v>314.00</v>
       </c>
       <c r="G104" t="str">
         <v>0.00</v>
       </c>
       <c r="H104" t="str">
-        <v>35940.64</v>
+        <v>36066.64</v>
       </c>
     </row>
     <row r="105">
@@ -2998,25 +2998,25 @@
         <v>99</v>
       </c>
       <c r="B105" t="str">
-        <v>19/08/2026</v>
+        <v>20/08/2026</v>
       </c>
       <c r="C105" t="str">
-        <v>19/08/2026</v>
+        <v>20/08/2026</v>
       </c>
       <c r="D105" t="str">
         <v>-</v>
       </c>
       <c r="E105" t="str">
-        <v>UPI/647575913695/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/658707792731/JIO PREPAID/jio@sbi/HDFC BANK</v>
       </c>
       <c r="F105" t="str">
-        <v>397.00</v>
+        <v>349.00</v>
       </c>
       <c r="G105" t="str">
         <v>0.00</v>
       </c>
       <c r="H105" t="str">
-        <v>35543.64</v>
+        <v>35717.64</v>
       </c>
     </row>
     <row r="106">
@@ -3024,25 +3024,25 @@
         <v>100</v>
       </c>
       <c r="B106" t="str">
-        <v>19/08/2026</v>
+        <v>20/08/2026</v>
       </c>
       <c r="C106" t="str">
-        <v>19/08/2026</v>
+        <v>20/08/2026</v>
       </c>
       <c r="D106" t="str">
         <v>-</v>
       </c>
       <c r="E106" t="str">
-        <v>UPI/388694588048/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/784573984984/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F106" t="str">
-        <v>548.00</v>
+        <v>430.00</v>
       </c>
       <c r="G106" t="str">
         <v>0.00</v>
       </c>
       <c r="H106" t="str">
-        <v>34995.64</v>
+        <v>35287.64</v>
       </c>
     </row>
     <row r="107">
@@ -3059,16 +3059,16 @@
         <v>-</v>
       </c>
       <c r="E107" t="str">
-        <v>UPI/915174024691/JIO PREPAID/jio@sbi/HDFC BANK</v>
+        <v>UPI/721649967506/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F107" t="str">
-        <v>349.00</v>
+        <v>452.00</v>
       </c>
       <c r="G107" t="str">
         <v>0.00</v>
       </c>
       <c r="H107" t="str">
-        <v>34646.64</v>
+        <v>34835.64</v>
       </c>
     </row>
     <row r="108">
@@ -3085,16 +3085,16 @@
         <v>-</v>
       </c>
       <c r="E108" t="str">
-        <v>UPI/583661613753/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/364485755702/AMRUTTULYA TEA/9716144905@paytm/HDFC BANK</v>
       </c>
       <c r="F108" t="str">
-        <v>159.00</v>
+        <v>111.00</v>
       </c>
       <c r="G108" t="str">
         <v>0.00</v>
       </c>
       <c r="H108" t="str">
-        <v>34487.64</v>
+        <v>34724.64</v>
       </c>
     </row>
     <row r="109">
@@ -3111,16 +3111,16 @@
         <v>-</v>
       </c>
       <c r="E109" t="str">
-        <v>UPI/233065250678/GOODLUCK CAFE/9706000585@paytm/HDFC BANK</v>
+        <v>UPI/234919467638/VAISHALI CAFE/9753740179@paytm/HDFC BANK</v>
       </c>
       <c r="F109" t="str">
-        <v>144.00</v>
+        <v>67.00</v>
       </c>
       <c r="G109" t="str">
         <v>0.00</v>
       </c>
       <c r="H109" t="str">
-        <v>34343.64</v>
+        <v>34657.64</v>
       </c>
     </row>
     <row r="110">
@@ -3137,16 +3137,16 @@
         <v>-</v>
       </c>
       <c r="E110" t="str">
-        <v>UPI/514681524760/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/820397937390/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F110" t="str">
-        <v>274.00</v>
+        <v>510.00</v>
       </c>
       <c r="G110" t="str">
         <v>0.00</v>
       </c>
       <c r="H110" t="str">
-        <v>34069.64</v>
+        <v>34147.64</v>
       </c>
     </row>
     <row r="111">
@@ -3163,16 +3163,16 @@
         <v>-</v>
       </c>
       <c r="E111" t="str">
-        <v>UPI/292604105593/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/480944083910/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F111" t="str">
-        <v>329.00</v>
+        <v>222.00</v>
       </c>
       <c r="G111" t="str">
         <v>0.00</v>
       </c>
       <c r="H111" t="str">
-        <v>33740.64</v>
+        <v>33925.64</v>
       </c>
     </row>
     <row r="112">
@@ -3180,25 +3180,25 @@
         <v>106</v>
       </c>
       <c r="B112" t="str">
-        <v>22/08/2026</v>
+        <v>23/08/2026</v>
       </c>
       <c r="C112" t="str">
-        <v>22/08/2026</v>
+        <v>23/08/2026</v>
       </c>
       <c r="D112" t="str">
         <v>-</v>
       </c>
       <c r="E112" t="str">
-        <v>UPI/189096809364/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/560592568526/VAISHALI CAFE/9755824221@paytm/HDFC BANK</v>
       </c>
       <c r="F112" t="str">
-        <v>141.00</v>
+        <v>184.00</v>
       </c>
       <c r="G112" t="str">
         <v>0.00</v>
       </c>
       <c r="H112" t="str">
-        <v>33599.64</v>
+        <v>33741.64</v>
       </c>
     </row>
     <row r="113">
@@ -3206,25 +3206,25 @@
         <v>107</v>
       </c>
       <c r="B113" t="str">
-        <v>22/08/2026</v>
+        <v>24/08/2026</v>
       </c>
       <c r="C113" t="str">
-        <v>22/08/2026</v>
+        <v>24/08/2026</v>
       </c>
       <c r="D113" t="str">
         <v>-</v>
       </c>
       <c r="E113" t="str">
-        <v>UPI/709191570570/PUNE PRINTS/9787898919@paytm/HDFC BANK</v>
+        <v>UPI/841506048943/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F113" t="str">
-        <v>55.00</v>
+        <v>2284.00</v>
       </c>
       <c r="G113" t="str">
         <v>0.00</v>
       </c>
       <c r="H113" t="str">
-        <v>33544.64</v>
+        <v>31457.64</v>
       </c>
     </row>
     <row r="114">
@@ -3232,25 +3232,25 @@
         <v>108</v>
       </c>
       <c r="B114" t="str">
-        <v>23/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="C114" t="str">
-        <v>23/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="D114" t="str">
         <v>-</v>
       </c>
       <c r="E114" t="str">
-        <v>UPI/590140748629/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/676390396896/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F114" t="str">
-        <v>500.00</v>
+        <v>412.00</v>
       </c>
       <c r="G114" t="str">
         <v>0.00</v>
       </c>
       <c r="H114" t="str">
-        <v>33044.64</v>
+        <v>31045.64</v>
       </c>
     </row>
     <row r="115">
@@ -3258,25 +3258,25 @@
         <v>109</v>
       </c>
       <c r="B115" t="str">
-        <v>23/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="C115" t="str">
-        <v>23/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="D115" t="str">
         <v>-</v>
       </c>
       <c r="E115" t="str">
-        <v>UPI/137788742803/AMRUTTULYA TEA/9703422257@paytm/HDFC BANK</v>
+        <v>UPI/697988076554/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F115" t="str">
-        <v>108.00</v>
+        <v>130.00</v>
       </c>
       <c r="G115" t="str">
         <v>0.00</v>
       </c>
       <c r="H115" t="str">
-        <v>32936.64</v>
+        <v>30915.64</v>
       </c>
     </row>
     <row r="116">
@@ -3284,25 +3284,25 @@
         <v>110</v>
       </c>
       <c r="B116" t="str">
-        <v>24/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="C116" t="str">
-        <v>24/08/2026</v>
+        <v>25/08/2026</v>
       </c>
       <c r="D116" t="str">
         <v>-</v>
       </c>
       <c r="E116" t="str">
-        <v>UPI/255287416279/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/804922614386/AMRUTTULYA TEA/9717468134@paytm/HDFC BANK</v>
       </c>
       <c r="F116" t="str">
-        <v>2034.00</v>
+        <v>50.00</v>
       </c>
       <c r="G116" t="str">
         <v>0.00</v>
       </c>
       <c r="H116" t="str">
-        <v>30902.64</v>
+        <v>30865.64</v>
       </c>
     </row>
     <row r="117">
@@ -3319,16 +3319,16 @@
         <v>-</v>
       </c>
       <c r="E117" t="str">
-        <v>UPI/991532637248/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/825344346347/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F117" t="str">
-        <v>606.00</v>
+        <v>465.00</v>
       </c>
       <c r="G117" t="str">
         <v>0.00</v>
       </c>
       <c r="H117" t="str">
-        <v>30296.64</v>
+        <v>30400.64</v>
       </c>
     </row>
     <row r="118">
@@ -3345,16 +3345,16 @@
         <v>-</v>
       </c>
       <c r="E118" t="str">
-        <v>UPI/363641035882/AMRUTTULYA TEA/9729759110@paytm/HDFC BANK</v>
+        <v>UPI/657232627435/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F118" t="str">
-        <v>225.00</v>
+        <v>469.00</v>
       </c>
       <c r="G118" t="str">
         <v>0.00</v>
       </c>
       <c r="H118" t="str">
-        <v>30071.64</v>
+        <v>29931.64</v>
       </c>
     </row>
     <row r="119">
@@ -3380,7 +3380,7 @@
         <v>54000.00</v>
       </c>
       <c r="H119" t="str">
-        <v>84071.64</v>
+        <v>83931.64</v>
       </c>
     </row>
     <row r="120">
@@ -3406,7 +3406,7 @@
         <v>0.00</v>
       </c>
       <c r="H120" t="str">
-        <v>83717.64</v>
+        <v>83577.64</v>
       </c>
     </row>
     <row r="121">
@@ -3423,7 +3423,7 @@
         <v>-</v>
       </c>
       <c r="E121" t="str">
-        <v>UPI/262071845424/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
+        <v>UPI/424781054956/OPENAI CHATGPT/openai@icici/HDFC BANK</v>
       </c>
       <c r="F121" t="str">
         <v>1999.00</v>
@@ -3432,7 +3432,7 @@
         <v>0.00</v>
       </c>
       <c r="H121" t="str">
-        <v>81718.64</v>
+        <v>81578.64</v>
       </c>
     </row>
     <row r="122">
@@ -3440,25 +3440,25 @@
         <v>116</v>
       </c>
       <c r="B122" t="str">
-        <v>03/09/2026</v>
+        <v>02/09/2026</v>
       </c>
       <c r="C122" t="str">
-        <v>03/09/2026</v>
+        <v>02/09/2026</v>
       </c>
       <c r="D122" t="str">
         <v>-</v>
       </c>
       <c r="E122" t="str">
-        <v>UPI/313382032606/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
+        <v>UPI/451120384153/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F122" t="str">
-        <v>1675.28</v>
+        <v>553.00</v>
       </c>
       <c r="G122" t="str">
         <v>0.00</v>
       </c>
       <c r="H122" t="str">
-        <v>80043.36</v>
+        <v>81025.64</v>
       </c>
     </row>
     <row r="123">
@@ -3466,25 +3466,25 @@
         <v>117</v>
       </c>
       <c r="B123" t="str">
-        <v>03/09/2026</v>
+        <v>02/09/2026</v>
       </c>
       <c r="C123" t="str">
-        <v>03/09/2026</v>
+        <v>02/09/2026</v>
       </c>
       <c r="D123" t="str">
         <v>-</v>
       </c>
       <c r="E123" t="str">
-        <v>UPI/504622609587/DMART/grocery@ybl/HDFC BANK</v>
+        <v>UPI/934469919116/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F123" t="str">
-        <v>945.00</v>
+        <v>378.00</v>
       </c>
       <c r="G123" t="str">
         <v>0.00</v>
       </c>
       <c r="H123" t="str">
-        <v>79098.36</v>
+        <v>80647.64</v>
       </c>
     </row>
     <row r="124">
@@ -3501,16 +3501,16 @@
         <v>-</v>
       </c>
       <c r="E124" t="str">
-        <v>UPI/581330053694/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/797660261904/ADOBE SYSTEMS/adobe@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F124" t="str">
-        <v>357.00</v>
+        <v>1675.28</v>
       </c>
       <c r="G124" t="str">
         <v>0.00</v>
       </c>
       <c r="H124" t="str">
-        <v>78741.36</v>
+        <v>78972.36</v>
       </c>
     </row>
     <row r="125">
@@ -3518,25 +3518,25 @@
         <v>119</v>
       </c>
       <c r="B125" t="str">
-        <v>04/09/2026</v>
+        <v>03/09/2026</v>
       </c>
       <c r="C125" t="str">
-        <v>04/09/2026</v>
+        <v>03/09/2026</v>
       </c>
       <c r="D125" t="str">
         <v>-</v>
       </c>
       <c r="E125" t="str">
-        <v>UPI/400784864998/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/627633096650/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F125" t="str">
-        <v>468.00</v>
+        <v>1407.00</v>
       </c>
       <c r="G125" t="str">
         <v>0.00</v>
       </c>
       <c r="H125" t="str">
-        <v>78273.36</v>
+        <v>77565.36</v>
       </c>
     </row>
     <row r="126">
@@ -3544,25 +3544,25 @@
         <v>120</v>
       </c>
       <c r="B126" t="str">
-        <v>04/09/2026</v>
+        <v>03/09/2026</v>
       </c>
       <c r="C126" t="str">
-        <v>04/09/2026</v>
+        <v>03/09/2026</v>
       </c>
       <c r="D126" t="str">
         <v>-</v>
       </c>
       <c r="E126" t="str">
-        <v>UPI/491802540654/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/265879785735/GOODLUCK CAFE/9735303004@paytm/HDFC BANK</v>
       </c>
       <c r="F126" t="str">
-        <v>532.00</v>
+        <v>196.00</v>
       </c>
       <c r="G126" t="str">
         <v>0.00</v>
       </c>
       <c r="H126" t="str">
-        <v>77741.36</v>
+        <v>77369.36</v>
       </c>
     </row>
     <row r="127">
@@ -3579,16 +3579,16 @@
         <v>-</v>
       </c>
       <c r="E127" t="str">
-        <v>UPI/432084345491/VAISHALI CAFE/9771166023@paytm/HDFC BANK</v>
+        <v>UPI/933129369700/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F127" t="str">
-        <v>59.00</v>
+        <v>326.00</v>
       </c>
       <c r="G127" t="str">
         <v>0.00</v>
       </c>
       <c r="H127" t="str">
-        <v>77682.36</v>
+        <v>77043.36</v>
       </c>
     </row>
     <row r="128">
@@ -3605,7 +3605,7 @@
         <v>-</v>
       </c>
       <c r="E128" t="str">
-        <v>MMT/IMPS/527275711880/Rent Sep/Meera Kulkarni/HDFC0001234</v>
+        <v>MMT/IMPS/273135990300/Rent Sep/Meera Kulkarni/HDFC0001234</v>
       </c>
       <c r="F128" t="str">
         <v>18500.00</v>
@@ -3614,7 +3614,7 @@
         <v>0.00</v>
       </c>
       <c r="H128" t="str">
-        <v>59182.36</v>
+        <v>58543.36</v>
       </c>
     </row>
     <row r="129">
@@ -3622,25 +3622,25 @@
         <v>123</v>
       </c>
       <c r="B129" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="C129" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="D129" t="str">
         <v>-</v>
       </c>
       <c r="E129" t="str">
-        <v>UPI/511963050812/NOTION LABS/notion@icici/HDFC BANK</v>
+        <v>UPI/612524485262/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F129" t="str">
-        <v>880.00</v>
+        <v>475.00</v>
       </c>
       <c r="G129" t="str">
         <v>0.00</v>
       </c>
       <c r="H129" t="str">
-        <v>58302.36</v>
+        <v>58068.36</v>
       </c>
     </row>
     <row r="130">
@@ -3648,25 +3648,25 @@
         <v>124</v>
       </c>
       <c r="B130" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="C130" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="D130" t="str">
         <v>-</v>
       </c>
       <c r="E130" t="str">
-        <v>UPI/755136693688/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/520358089474/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F130" t="str">
-        <v>651.00</v>
+        <v>325.00</v>
       </c>
       <c r="G130" t="str">
         <v>0.00</v>
       </c>
       <c r="H130" t="str">
-        <v>57651.36</v>
+        <v>57743.36</v>
       </c>
     </row>
     <row r="131">
@@ -3674,25 +3674,25 @@
         <v>125</v>
       </c>
       <c r="B131" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="C131" t="str">
-        <v>06/09/2026</v>
+        <v>05/09/2026</v>
       </c>
       <c r="D131" t="str">
         <v>-</v>
       </c>
       <c r="E131" t="str">
-        <v>UPI/409059412125/AMRUTTULYA TEA/9756179768@paytm/HDFC BANK</v>
+        <v>UPI/175281596882/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F131" t="str">
-        <v>149.00</v>
+        <v>187.00</v>
       </c>
       <c r="G131" t="str">
         <v>0.00</v>
       </c>
       <c r="H131" t="str">
-        <v>57502.36</v>
+        <v>57556.36</v>
       </c>
     </row>
     <row r="132">
@@ -3700,25 +3700,25 @@
         <v>126</v>
       </c>
       <c r="B132" t="str">
-        <v>07/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="C132" t="str">
-        <v>07/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="D132" t="str">
         <v>-</v>
       </c>
       <c r="E132" t="str">
-        <v>UPI/253569855564/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/657125235768/NOTION LABS/notion@icici/HDFC BANK</v>
       </c>
       <c r="F132" t="str">
-        <v>471.00</v>
+        <v>880.00</v>
       </c>
       <c r="G132" t="str">
         <v>0.00</v>
       </c>
       <c r="H132" t="str">
-        <v>57031.36</v>
+        <v>56676.36</v>
       </c>
     </row>
     <row r="133">
@@ -3726,25 +3726,25 @@
         <v>127</v>
       </c>
       <c r="B133" t="str">
-        <v>08/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="C133" t="str">
-        <v>08/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="D133" t="str">
         <v>-</v>
       </c>
       <c r="E133" t="str">
-        <v>UPI/813739177701/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
+        <v>UPI/165050003817/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F133" t="str">
-        <v>1567.00</v>
+        <v>316.00</v>
       </c>
       <c r="G133" t="str">
         <v>0.00</v>
       </c>
       <c r="H133" t="str">
-        <v>55464.36</v>
+        <v>56360.36</v>
       </c>
     </row>
     <row r="134">
@@ -3752,25 +3752,25 @@
         <v>128</v>
       </c>
       <c r="B134" t="str">
-        <v>08/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="C134" t="str">
-        <v>08/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="D134" t="str">
         <v>-</v>
       </c>
       <c r="E134" t="str">
-        <v>UPI/544931887695/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/525408118451/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F134" t="str">
-        <v>343.00</v>
+        <v>495.00</v>
       </c>
       <c r="G134" t="str">
         <v>0.00</v>
       </c>
       <c r="H134" t="str">
-        <v>55121.36</v>
+        <v>55865.36</v>
       </c>
     </row>
     <row r="135">
@@ -3778,25 +3778,25 @@
         <v>129</v>
       </c>
       <c r="B135" t="str">
-        <v>10/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="C135" t="str">
-        <v>10/09/2026</v>
+        <v>06/09/2026</v>
       </c>
       <c r="D135" t="str">
         <v>-</v>
       </c>
       <c r="E135" t="str">
-        <v>UPI/526966667547/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
+        <v>UPI/335336561314/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F135" t="str">
-        <v>119.00</v>
+        <v>530.00</v>
       </c>
       <c r="G135" t="str">
         <v>0.00</v>
       </c>
       <c r="H135" t="str">
-        <v>55002.36</v>
+        <v>55335.36</v>
       </c>
     </row>
     <row r="136">
@@ -3804,25 +3804,25 @@
         <v>130</v>
       </c>
       <c r="B136" t="str">
-        <v>10/09/2026</v>
+        <v>07/09/2026</v>
       </c>
       <c r="C136" t="str">
-        <v>10/09/2026</v>
+        <v>07/09/2026</v>
       </c>
       <c r="D136" t="str">
         <v>-</v>
       </c>
       <c r="E136" t="str">
-        <v>UPI/418169628921/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/511963050812/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F136" t="str">
-        <v>441.00</v>
+        <v>571.00</v>
       </c>
       <c r="G136" t="str">
         <v>0.00</v>
       </c>
       <c r="H136" t="str">
-        <v>54561.36</v>
+        <v>54764.36</v>
       </c>
     </row>
     <row r="137">
@@ -3830,25 +3830,25 @@
         <v>131</v>
       </c>
       <c r="B137" t="str">
-        <v>10/09/2026</v>
+        <v>07/09/2026</v>
       </c>
       <c r="C137" t="str">
-        <v>10/09/2026</v>
+        <v>07/09/2026</v>
       </c>
       <c r="D137" t="str">
         <v>-</v>
       </c>
       <c r="E137" t="str">
-        <v>UPI/973619440849/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/418169628921/AMRUTTULYA TEA/9721674655@paytm/HDFC BANK</v>
       </c>
       <c r="F137" t="str">
-        <v>1077.00</v>
+        <v>134.00</v>
       </c>
       <c r="G137" t="str">
         <v>0.00</v>
       </c>
       <c r="H137" t="str">
-        <v>53484.36</v>
+        <v>54630.36</v>
       </c>
     </row>
     <row r="138">
@@ -3856,25 +3856,25 @@
         <v>132</v>
       </c>
       <c r="B138" t="str">
-        <v>11/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="C138" t="str">
-        <v>11/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="D138" t="str">
         <v>-</v>
       </c>
       <c r="E138" t="str">
-        <v>UPI/187358679668/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/305593053321/LINKEDIN PREMIUM/linkedin@icici/HDFC BANK</v>
       </c>
       <c r="F138" t="str">
-        <v>521.00</v>
+        <v>1567.00</v>
       </c>
       <c r="G138" t="str">
         <v>0.00</v>
       </c>
       <c r="H138" t="str">
-        <v>52963.36</v>
+        <v>53063.36</v>
       </c>
     </row>
     <row r="139">
@@ -3882,25 +3882,25 @@
         <v>133</v>
       </c>
       <c r="B139" t="str">
-        <v>11/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="C139" t="str">
-        <v>11/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="D139" t="str">
         <v>-</v>
       </c>
       <c r="E139" t="str">
-        <v>UPI/800714295706/PUNE PRINTS/9759165624@paytm/HDFC BANK</v>
+        <v>UPI/370796784386/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F139" t="str">
-        <v>168.00</v>
+        <v>311.00</v>
       </c>
       <c r="G139" t="str">
         <v>0.00</v>
       </c>
       <c r="H139" t="str">
-        <v>52795.36</v>
+        <v>52752.36</v>
       </c>
     </row>
     <row r="140">
@@ -3908,25 +3908,25 @@
         <v>134</v>
       </c>
       <c r="B140" t="str">
-        <v>12/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="C140" t="str">
-        <v>12/09/2026</v>
+        <v>08/09/2026</v>
       </c>
       <c r="D140" t="str">
         <v>-</v>
       </c>
       <c r="E140" t="str">
-        <v>UPI/933129369700/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/544215664756/PUNE PRINTS/9718910817@paytm/HDFC BANK</v>
       </c>
       <c r="F140" t="str">
-        <v>570.00</v>
+        <v>162.00</v>
       </c>
       <c r="G140" t="str">
         <v>0.00</v>
       </c>
       <c r="H140" t="str">
-        <v>52225.36</v>
+        <v>52590.36</v>
       </c>
     </row>
     <row r="141">
@@ -3934,25 +3934,25 @@
         <v>135</v>
       </c>
       <c r="B141" t="str">
-        <v>12/09/2026</v>
+        <v>09/09/2026</v>
       </c>
       <c r="C141" t="str">
-        <v>12/09/2026</v>
+        <v>09/09/2026</v>
       </c>
       <c r="D141" t="str">
         <v>-</v>
       </c>
       <c r="E141" t="str">
-        <v>UPI/885168938036/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/976166544272/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F141" t="str">
-        <v>313.00</v>
+        <v>556.00</v>
       </c>
       <c r="G141" t="str">
         <v>0.00</v>
       </c>
       <c r="H141" t="str">
-        <v>51912.36</v>
+        <v>52034.36</v>
       </c>
     </row>
     <row r="142">
@@ -3960,25 +3960,25 @@
         <v>136</v>
       </c>
       <c r="B142" t="str">
-        <v>12/09/2026</v>
+        <v>09/09/2026</v>
       </c>
       <c r="C142" t="str">
-        <v>12/09/2026</v>
+        <v>09/09/2026</v>
       </c>
       <c r="D142" t="str">
         <v>-</v>
       </c>
       <c r="E142" t="str">
-        <v>UPI/264988920185/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/464734385488/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F142" t="str">
-        <v>220.00</v>
+        <v>327.00</v>
       </c>
       <c r="G142" t="str">
         <v>0.00</v>
       </c>
       <c r="H142" t="str">
-        <v>51692.36</v>
+        <v>51707.36</v>
       </c>
     </row>
     <row r="143">
@@ -3986,25 +3986,25 @@
         <v>137</v>
       </c>
       <c r="B143" t="str">
-        <v>12/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="C143" t="str">
-        <v>12/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="D143" t="str">
         <v>-</v>
       </c>
       <c r="E143" t="str">
-        <v>UPI/353407947695/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/853475504321/SPOTIFY INDIA/spotify@axisbank/HDFC BANK</v>
       </c>
       <c r="F143" t="str">
-        <v>233.00</v>
+        <v>119.00</v>
       </c>
       <c r="G143" t="str">
         <v>0.00</v>
       </c>
       <c r="H143" t="str">
-        <v>51459.36</v>
+        <v>51588.36</v>
       </c>
     </row>
     <row r="144">
@@ -4012,25 +4012,25 @@
         <v>138</v>
       </c>
       <c r="B144" t="str">
-        <v>12/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="C144" t="str">
-        <v>12/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="D144" t="str">
         <v>-</v>
       </c>
       <c r="E144" t="str">
-        <v>ATM CASH WDL ATW 661021 PUNE FC ROAD</v>
+        <v>UPI/621028234274/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F144" t="str">
-        <v>3000.00</v>
+        <v>454.00</v>
       </c>
       <c r="G144" t="str">
         <v>0.00</v>
       </c>
       <c r="H144" t="str">
-        <v>48459.36</v>
+        <v>51134.36</v>
       </c>
     </row>
     <row r="145">
@@ -4038,25 +4038,25 @@
         <v>139</v>
       </c>
       <c r="B145" t="str">
-        <v>13/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="C145" t="str">
-        <v>13/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="D145" t="str">
         <v>-</v>
       </c>
       <c r="E145" t="str">
-        <v>UPI/605505367857/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
+        <v>UPI/809923724271/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F145" t="str">
-        <v>299.00</v>
+        <v>369.00</v>
       </c>
       <c r="G145" t="str">
         <v>0.00</v>
       </c>
       <c r="H145" t="str">
-        <v>48160.36</v>
+        <v>50765.36</v>
       </c>
     </row>
     <row r="146">
@@ -4064,25 +4064,25 @@
         <v>140</v>
       </c>
       <c r="B146" t="str">
-        <v>13/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="C146" t="str">
-        <v>13/09/2026</v>
+        <v>10/09/2026</v>
       </c>
       <c r="D146" t="str">
         <v>-</v>
       </c>
       <c r="E146" t="str">
-        <v>UPI/581211043661/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
+        <v>UPI/211950590345/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F146" t="str">
-        <v>299.00</v>
+        <v>1046.00</v>
       </c>
       <c r="G146" t="str">
         <v>0.00</v>
       </c>
       <c r="H146" t="str">
-        <v>47861.36</v>
+        <v>49719.36</v>
       </c>
     </row>
     <row r="147">
@@ -4090,25 +4090,25 @@
         <v>141</v>
       </c>
       <c r="B147" t="str">
-        <v>13/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="C147" t="str">
-        <v>13/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="D147" t="str">
         <v>-</v>
       </c>
       <c r="E147" t="str">
-        <v>UPI/198569640284/PUNE PRINTS/9724292975@paytm/HDFC BANK</v>
+        <v>UPI/927556488499/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F147" t="str">
-        <v>145.00</v>
+        <v>447.00</v>
       </c>
       <c r="G147" t="str">
         <v>0.00</v>
       </c>
       <c r="H147" t="str">
-        <v>47716.36</v>
+        <v>49272.36</v>
       </c>
     </row>
     <row r="148">
@@ -4116,25 +4116,25 @@
         <v>142</v>
       </c>
       <c r="B148" t="str">
-        <v>14/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="C148" t="str">
-        <v>14/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="D148" t="str">
         <v>-</v>
       </c>
       <c r="E148" t="str">
-        <v>UPI/597259495430/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/762743546371/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F148" t="str">
-        <v>518.00</v>
+        <v>249.00</v>
       </c>
       <c r="G148" t="str">
         <v>0.00</v>
       </c>
       <c r="H148" t="str">
-        <v>47198.36</v>
+        <v>49023.36</v>
       </c>
     </row>
     <row r="149">
@@ -4142,25 +4142,25 @@
         <v>143</v>
       </c>
       <c r="B149" t="str">
-        <v>14/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="C149" t="str">
-        <v>14/09/2026</v>
+        <v>11/09/2026</v>
       </c>
       <c r="D149" t="str">
         <v>-</v>
       </c>
       <c r="E149" t="str">
-        <v>UPI/210840115370/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/667711286735/VAISHALI CAFE/9726113025@paytm/HDFC BANK</v>
       </c>
       <c r="F149" t="str">
-        <v>213.00</v>
+        <v>74.00</v>
       </c>
       <c r="G149" t="str">
         <v>0.00</v>
       </c>
       <c r="H149" t="str">
-        <v>46985.36</v>
+        <v>48949.36</v>
       </c>
     </row>
     <row r="150">
@@ -4168,25 +4168,25 @@
         <v>144</v>
       </c>
       <c r="B150" t="str">
-        <v>15/09/2026</v>
+        <v>12/09/2026</v>
       </c>
       <c r="C150" t="str">
-        <v>15/09/2026</v>
+        <v>12/09/2026</v>
       </c>
       <c r="D150" t="str">
         <v>-</v>
       </c>
       <c r="E150" t="str">
-        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/310508435</v>
+        <v>UPI/455906429281/AMRUTTULYA TEA/9710142960@paytm/HDFC BANK</v>
       </c>
       <c r="F150" t="str">
-        <v>4210.00</v>
+        <v>204.00</v>
       </c>
       <c r="G150" t="str">
         <v>0.00</v>
       </c>
       <c r="H150" t="str">
-        <v>42775.36</v>
+        <v>48745.36</v>
       </c>
     </row>
     <row r="151">
@@ -4194,25 +4194,25 @@
         <v>145</v>
       </c>
       <c r="B151" t="str">
-        <v>15/09/2026</v>
+        <v>12/09/2026</v>
       </c>
       <c r="C151" t="str">
-        <v>15/09/2026</v>
+        <v>12/09/2026</v>
       </c>
       <c r="D151" t="str">
         <v>-</v>
       </c>
       <c r="E151" t="str">
-        <v>UPI/266701188776/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>ATM CASH WDL ATW 504622 PUNE FC ROAD</v>
       </c>
       <c r="F151" t="str">
-        <v>316.00</v>
+        <v>3000.00</v>
       </c>
       <c r="G151" t="str">
         <v>0.00</v>
       </c>
       <c r="H151" t="str">
-        <v>42459.36</v>
+        <v>45745.36</v>
       </c>
     </row>
     <row r="152">
@@ -4220,25 +4220,25 @@
         <v>146</v>
       </c>
       <c r="B152" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="C152" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="D152" t="str">
         <v>-</v>
       </c>
       <c r="E152" t="str">
-        <v>UPI/809923724271/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/337549306219/JIOHOTSTAR/jiohotstar@ybl/HDFC BANK</v>
       </c>
       <c r="F152" t="str">
-        <v>369.00</v>
+        <v>299.00</v>
       </c>
       <c r="G152" t="str">
         <v>0.00</v>
       </c>
       <c r="H152" t="str">
-        <v>42090.36</v>
+        <v>45446.36</v>
       </c>
     </row>
     <row r="153">
@@ -4246,25 +4246,25 @@
         <v>147</v>
       </c>
       <c r="B153" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="C153" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="D153" t="str">
         <v>-</v>
       </c>
       <c r="E153" t="str">
-        <v>UPI/255058220471/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/437316836975/SONYLIV/sonyliv@hdfcbank/HDFC BANK</v>
       </c>
       <c r="F153" t="str">
-        <v>554.00</v>
+        <v>299.00</v>
       </c>
       <c r="G153" t="str">
         <v>0.00</v>
       </c>
       <c r="H153" t="str">
-        <v>41536.36</v>
+        <v>45147.36</v>
       </c>
     </row>
     <row r="154">
@@ -4272,25 +4272,25 @@
         <v>148</v>
       </c>
       <c r="B154" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="C154" t="str">
-        <v>16/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="D154" t="str">
         <v>-</v>
       </c>
       <c r="E154" t="str">
-        <v>UPI/264126996719/GOODLUCK CAFE/9731189034@paytm/HDFC BANK</v>
+        <v>UPI/720284099085/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F154" t="str">
-        <v>229.00</v>
+        <v>452.00</v>
       </c>
       <c r="G154" t="str">
         <v>0.00</v>
       </c>
       <c r="H154" t="str">
-        <v>41307.36</v>
+        <v>44695.36</v>
       </c>
     </row>
     <row r="155">
@@ -4298,25 +4298,25 @@
         <v>149</v>
       </c>
       <c r="B155" t="str">
-        <v>17/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="C155" t="str">
-        <v>17/09/2026</v>
+        <v>13/09/2026</v>
       </c>
       <c r="D155" t="str">
         <v>-</v>
       </c>
       <c r="E155" t="str">
-        <v>UPI/503504010871/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
+        <v>UPI/848476292309/PUNE PRINTS/9771342621@paytm/HDFC BANK</v>
       </c>
       <c r="F155" t="str">
-        <v>1445.00</v>
+        <v>186.00</v>
       </c>
       <c r="G155" t="str">
         <v>0.00</v>
       </c>
       <c r="H155" t="str">
-        <v>39862.36</v>
+        <v>44509.36</v>
       </c>
     </row>
     <row r="156">
@@ -4324,25 +4324,25 @@
         <v>150</v>
       </c>
       <c r="B156" t="str">
-        <v>17/09/2026</v>
+        <v>15/09/2026</v>
       </c>
       <c r="C156" t="str">
-        <v>17/09/2026</v>
+        <v>15/09/2026</v>
       </c>
       <c r="D156" t="str">
         <v>-</v>
       </c>
       <c r="E156" t="str">
-        <v>UPI/451716545969/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>ACH/BAJAJ FINANCE LTD/EMI LAPTOP/392727048</v>
       </c>
       <c r="F156" t="str">
-        <v>602.00</v>
+        <v>4210.00</v>
       </c>
       <c r="G156" t="str">
         <v>0.00</v>
       </c>
       <c r="H156" t="str">
-        <v>39260.36</v>
+        <v>40299.36</v>
       </c>
     </row>
     <row r="157">
@@ -4350,25 +4350,25 @@
         <v>151</v>
       </c>
       <c r="B157" t="str">
-        <v>17/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="C157" t="str">
-        <v>17/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="D157" t="str">
         <v>-</v>
       </c>
       <c r="E157" t="str">
-        <v>UPI/173879066645/DMART/grocery@ybl/HDFC BANK</v>
+        <v>UPI/581211043661/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F157" t="str">
-        <v>746.00</v>
+        <v>418.00</v>
       </c>
       <c r="G157" t="str">
         <v>0.00</v>
       </c>
       <c r="H157" t="str">
-        <v>38514.36</v>
+        <v>39881.36</v>
       </c>
     </row>
     <row r="158">
@@ -4376,25 +4376,25 @@
         <v>152</v>
       </c>
       <c r="B158" t="str">
-        <v>17/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="C158" t="str">
-        <v>17/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="D158" t="str">
         <v>-</v>
       </c>
       <c r="E158" t="str">
-        <v>UPI/456324083800/AMRUTTULYA TEA/9754920129@paytm/HDFC BANK</v>
+        <v>UPI/127441691118/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F158" t="str">
-        <v>97.00</v>
+        <v>272.00</v>
       </c>
       <c r="G158" t="str">
         <v>0.00</v>
       </c>
       <c r="H158" t="str">
-        <v>38417.36</v>
+        <v>39609.36</v>
       </c>
     </row>
     <row r="159">
@@ -4402,25 +4402,25 @@
         <v>153</v>
       </c>
       <c r="B159" t="str">
-        <v>18/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="C159" t="str">
-        <v>18/09/2026</v>
+        <v>16/09/2026</v>
       </c>
       <c r="D159" t="str">
         <v>-</v>
       </c>
       <c r="E159" t="str">
-        <v>UPI/540881603094/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/939552376000/VAISHALI CAFE/9769333298@paytm/HDFC BANK</v>
       </c>
       <c r="F159" t="str">
-        <v>268.00</v>
+        <v>64.00</v>
       </c>
       <c r="G159" t="str">
         <v>0.00</v>
       </c>
       <c r="H159" t="str">
-        <v>38149.36</v>
+        <v>39545.36</v>
       </c>
     </row>
     <row r="160">
@@ -4428,25 +4428,25 @@
         <v>154</v>
       </c>
       <c r="B160" t="str">
-        <v>18/09/2026</v>
+        <v>17/09/2026</v>
       </c>
       <c r="C160" t="str">
-        <v>18/09/2026</v>
+        <v>17/09/2026</v>
       </c>
       <c r="D160" t="str">
         <v>-</v>
       </c>
       <c r="E160" t="str">
-        <v>UPI/968103953055/AMRUTTULYA TEA/9704796227@paytm/HDFC BANK</v>
+        <v>UPI/540286793489/MSEDCL ELECTRICITY/msedcl@sbi/HDFC BANK</v>
       </c>
       <c r="F160" t="str">
-        <v>60.00</v>
+        <v>1370.00</v>
       </c>
       <c r="G160" t="str">
         <v>0.00</v>
       </c>
       <c r="H160" t="str">
-        <v>38089.36</v>
+        <v>38175.36</v>
       </c>
     </row>
     <row r="161">
@@ -4454,25 +4454,25 @@
         <v>155</v>
       </c>
       <c r="B161" t="str">
-        <v>18/09/2026</v>
+        <v>17/09/2026</v>
       </c>
       <c r="C161" t="str">
-        <v>18/09/2026</v>
+        <v>17/09/2026</v>
       </c>
       <c r="D161" t="str">
         <v>-</v>
       </c>
       <c r="E161" t="str">
-        <v>UPI/242736621224/BOOKMYSHOW/bookmyshow@icici/HDFC BANK</v>
+        <v>UPI/597259495430/DMART/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F161" t="str">
-        <v>760.00</v>
+        <v>1762.00</v>
       </c>
       <c r="G161" t="str">
         <v>0.00</v>
       </c>
       <c r="H161" t="str">
-        <v>37329.36</v>
+        <v>36413.36</v>
       </c>
     </row>
     <row r="162">
@@ -4489,16 +4489,16 @@
         <v>-</v>
       </c>
       <c r="E162" t="str">
-        <v>UPI/184720314922/BOOKMYSHOW/bookmyshow@icici/HDFC BANK</v>
+        <v>UPI/246925548580/VAISHALI CAFE/9748986844@paytm/HDFC BANK</v>
       </c>
       <c r="F162" t="str">
-        <v>760.00</v>
+        <v>96.00</v>
       </c>
       <c r="G162" t="str">
         <v>0.00</v>
       </c>
       <c r="H162" t="str">
-        <v>36569.36</v>
+        <v>36317.36</v>
       </c>
     </row>
     <row r="163">
@@ -4506,25 +4506,25 @@
         <v>157</v>
       </c>
       <c r="B163" t="str">
-        <v>19/09/2026</v>
+        <v>18/09/2026</v>
       </c>
       <c r="C163" t="str">
-        <v>19/09/2026</v>
+        <v>18/09/2026</v>
       </c>
       <c r="D163" t="str">
         <v>-</v>
       </c>
       <c r="E163" t="str">
-        <v>UPI/976170161482/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/282514619734/BOOKMYSHOW/bookmyshow@icici/HDFC BANK</v>
       </c>
       <c r="F163" t="str">
-        <v>245.00</v>
+        <v>760.00</v>
       </c>
       <c r="G163" t="str">
         <v>0.00</v>
       </c>
       <c r="H163" t="str">
-        <v>36324.36</v>
+        <v>35557.36</v>
       </c>
     </row>
     <row r="164">
@@ -4532,25 +4532,25 @@
         <v>158</v>
       </c>
       <c r="B164" t="str">
-        <v>20/09/2026</v>
+        <v>18/09/2026</v>
       </c>
       <c r="C164" t="str">
-        <v>20/09/2026</v>
+        <v>18/09/2026</v>
       </c>
       <c r="D164" t="str">
         <v>-</v>
       </c>
       <c r="E164" t="str">
-        <v>UPI/591077799093/JIO PREPAID/jio@sbi/HDFC BANK</v>
+        <v>UPI/973619440849/BOOKMYSHOW/bookmyshow@icici/HDFC BANK</v>
       </c>
       <c r="F164" t="str">
-        <v>349.00</v>
+        <v>760.00</v>
       </c>
       <c r="G164" t="str">
         <v>0.00</v>
       </c>
       <c r="H164" t="str">
-        <v>35975.36</v>
+        <v>34797.36</v>
       </c>
     </row>
     <row r="165">
@@ -4558,25 +4558,25 @@
         <v>159</v>
       </c>
       <c r="B165" t="str">
-        <v>20/09/2026</v>
+        <v>19/09/2026</v>
       </c>
       <c r="C165" t="str">
-        <v>20/09/2026</v>
+        <v>19/09/2026</v>
       </c>
       <c r="D165" t="str">
         <v>-</v>
       </c>
       <c r="E165" t="str">
-        <v>UPI/520358089474/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/210998321487/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F165" t="str">
-        <v>325.00</v>
+        <v>548.00</v>
       </c>
       <c r="G165" t="str">
         <v>0.00</v>
       </c>
       <c r="H165" t="str">
-        <v>35650.36</v>
+        <v>34249.36</v>
       </c>
     </row>
     <row r="166">
@@ -4584,25 +4584,25 @@
         <v>160</v>
       </c>
       <c r="B166" t="str">
-        <v>21/09/2026</v>
+        <v>20/09/2026</v>
       </c>
       <c r="C166" t="str">
-        <v>21/09/2026</v>
+        <v>20/09/2026</v>
       </c>
       <c r="D166" t="str">
         <v>-</v>
       </c>
       <c r="E166" t="str">
-        <v>UPI/986875357641/VAISHALI CAFE/9725209961@paytm/HDFC BANK</v>
+        <v>UPI/167674676515/JIO PREPAID/jio@sbi/HDFC BANK</v>
       </c>
       <c r="F166" t="str">
-        <v>32.00</v>
+        <v>349.00</v>
       </c>
       <c r="G166" t="str">
         <v>0.00</v>
       </c>
       <c r="H166" t="str">
-        <v>35618.36</v>
+        <v>33900.36</v>
       </c>
     </row>
     <row r="167">
@@ -4610,25 +4610,25 @@
         <v>161</v>
       </c>
       <c r="B167" t="str">
-        <v>21/09/2026</v>
+        <v>20/09/2026</v>
       </c>
       <c r="C167" t="str">
-        <v>21/09/2026</v>
+        <v>20/09/2026</v>
       </c>
       <c r="D167" t="str">
         <v>-</v>
       </c>
       <c r="E167" t="str">
-        <v>UPI/414203998399/VAISHALI CAFE/9774171641@paytm/HDFC BANK</v>
+        <v>UPI/202024840144/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F167" t="str">
-        <v>76.00</v>
+        <v>667.00</v>
       </c>
       <c r="G167" t="str">
         <v>0.00</v>
       </c>
       <c r="H167" t="str">
-        <v>35542.36</v>
+        <v>33233.36</v>
       </c>
     </row>
     <row r="168">
@@ -4636,25 +4636,25 @@
         <v>162</v>
       </c>
       <c r="B168" t="str">
-        <v>22/09/2026</v>
+        <v>21/09/2026</v>
       </c>
       <c r="C168" t="str">
-        <v>22/09/2026</v>
+        <v>21/09/2026</v>
       </c>
       <c r="D168" t="str">
         <v>-</v>
       </c>
       <c r="E168" t="str">
-        <v>IMPS-626512345678-KESTREL APPS-BKID-XXXXXXX0091-INVOICE</v>
+        <v>UPI/656903621810/GOODLUCK CAFE/9796010110@paytm/HDFC BANK</v>
       </c>
       <c r="F168" t="str">
-        <v>0.00</v>
+        <v>187.00</v>
       </c>
       <c r="G168" t="str">
-        <v>36500.00</v>
+        <v>0.00</v>
       </c>
       <c r="H168" t="str">
-        <v>72042.36</v>
+        <v>33046.36</v>
       </c>
     </row>
     <row r="169">
@@ -4671,16 +4671,16 @@
         <v>-</v>
       </c>
       <c r="E169" t="str">
-        <v>UPI/809215946518/GOODLUCK CAFE/9782890111@paytm/HDFC BANK</v>
+        <v>IMPS-626512345678-KESTREL APPS-BKID-XXXXXXX0091-INVOICE</v>
       </c>
       <c r="F169" t="str">
-        <v>127.00</v>
+        <v>0.00</v>
       </c>
       <c r="G169" t="str">
-        <v>0.00</v>
+        <v>36500.00</v>
       </c>
       <c r="H169" t="str">
-        <v>71915.36</v>
+        <v>69546.36</v>
       </c>
     </row>
     <row r="170">
@@ -4688,25 +4688,25 @@
         <v>164</v>
       </c>
       <c r="B170" t="str">
-        <v>24/09/2026</v>
+        <v>22/09/2026</v>
       </c>
       <c r="C170" t="str">
-        <v>24/09/2026</v>
+        <v>22/09/2026</v>
       </c>
       <c r="D170" t="str">
         <v>-</v>
       </c>
       <c r="E170" t="str">
-        <v>UPI/259657929185/ZOMATO/zomato@icici/HDFC BANK</v>
+        <v>UPI/799148755264/AMRUTTULYA TEA/9712682917@paytm/HDFC BANK</v>
       </c>
       <c r="F170" t="str">
-        <v>230.00</v>
+        <v>162.00</v>
       </c>
       <c r="G170" t="str">
         <v>0.00</v>
       </c>
       <c r="H170" t="str">
-        <v>71685.36</v>
+        <v>69384.36</v>
       </c>
     </row>
     <row r="171">
@@ -4714,25 +4714,25 @@
         <v>165</v>
       </c>
       <c r="B171" t="str">
-        <v>24/09/2026</v>
+        <v>23/09/2026</v>
       </c>
       <c r="C171" t="str">
-        <v>24/09/2026</v>
+        <v>23/09/2026</v>
       </c>
       <c r="D171" t="str">
         <v>-</v>
       </c>
       <c r="E171" t="str">
-        <v>UPI/417727036145/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/916518162190/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F171" t="str">
-        <v>278.00</v>
+        <v>584.00</v>
       </c>
       <c r="G171" t="str">
         <v>0.00</v>
       </c>
       <c r="H171" t="str">
-        <v>71407.36</v>
+        <v>68800.36</v>
       </c>
     </row>
     <row r="172">
@@ -4749,16 +4749,16 @@
         <v>-</v>
       </c>
       <c r="E172" t="str">
-        <v>UPI/667711286735/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/574951917608/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F172" t="str">
-        <v>295.00</v>
+        <v>514.00</v>
       </c>
       <c r="G172" t="str">
         <v>0.00</v>
       </c>
       <c r="H172" t="str">
-        <v>71112.36</v>
+        <v>68286.36</v>
       </c>
     </row>
     <row r="173">
@@ -4775,16 +4775,16 @@
         <v>-</v>
       </c>
       <c r="E173" t="str">
-        <v>UPI/280001880438/BLINKIT/grocery@ybl/HDFC BANK</v>
+        <v>UPI/925360005116/BLINKIT/grocery@ybl/HDFC BANK</v>
       </c>
       <c r="F173" t="str">
-        <v>2113.00</v>
+        <v>1909.00</v>
       </c>
       <c r="G173" t="str">
         <v>0.00</v>
       </c>
       <c r="H173" t="str">
-        <v>68999.36</v>
+        <v>66377.36</v>
       </c>
     </row>
     <row r="174">
@@ -4792,25 +4792,25 @@
         <v>168</v>
       </c>
       <c r="B174" t="str">
-        <v>26/09/2026</v>
+        <v>24/09/2026</v>
       </c>
       <c r="C174" t="str">
-        <v>26/09/2026</v>
+        <v>24/09/2026</v>
       </c>
       <c r="D174" t="str">
         <v>-</v>
       </c>
       <c r="E174" t="str">
-        <v>UPI/671833319379/SWIGGY/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/744802946387/UBER INDIA/uber@axisbank/HDFC BANK</v>
       </c>
       <c r="F174" t="str">
-        <v>571.00</v>
+        <v>341.00</v>
       </c>
       <c r="G174" t="str">
         <v>0.00</v>
       </c>
       <c r="H174" t="str">
-        <v>68428.36</v>
+        <v>66036.36</v>
       </c>
     </row>
     <row r="175">
@@ -4818,25 +4818,25 @@
         <v>169</v>
       </c>
       <c r="B175" t="str">
-        <v>26/09/2026</v>
+        <v>27/09/2026</v>
       </c>
       <c r="C175" t="str">
-        <v>26/09/2026</v>
+        <v>27/09/2026</v>
       </c>
       <c r="D175" t="str">
         <v>-</v>
       </c>
       <c r="E175" t="str">
-        <v>UPI/370796784386/ZOMATO/swiggy@ybl/HDFC BANK</v>
+        <v>UPI/720467709493/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F175" t="str">
-        <v>542.00</v>
+        <v>285.00</v>
       </c>
       <c r="G175" t="str">
         <v>0.00</v>
       </c>
       <c r="H175" t="str">
-        <v>67886.36</v>
+        <v>65751.36</v>
       </c>
     </row>
     <row r="176">
@@ -4844,25 +4844,25 @@
         <v>170</v>
       </c>
       <c r="B176" t="str">
-        <v>28/09/2026</v>
+        <v>27/09/2026</v>
       </c>
       <c r="C176" t="str">
-        <v>28/09/2026</v>
+        <v>27/09/2026</v>
       </c>
       <c r="D176" t="str">
         <v>-</v>
       </c>
       <c r="E176" t="str">
-        <v>UPI/796690595778/SWIGGY/zomato@icici/HDFC BANK</v>
+        <v>UPI/872277305042/SWIGGY/swiggy@ybl/HDFC BANK</v>
       </c>
       <c r="F176" t="str">
-        <v>595.00</v>
+        <v>635.00</v>
       </c>
       <c r="G176" t="str">
         <v>0.00</v>
       </c>
       <c r="H176" t="str">
-        <v>67291.36</v>
+        <v>65116.36</v>
       </c>
     </row>
     <row r="177">
@@ -4879,16 +4879,16 @@
         <v>-</v>
       </c>
       <c r="E177" t="str">
-        <v>UPI/657374288933/UBER INDIA/uber@axisbank/HDFC BANK</v>
+        <v>UPI/260266595333/ZOMATO/zomato@icici/HDFC BANK</v>
       </c>
       <c r="F177" t="str">
-        <v>340.00</v>
+        <v>448.00</v>
       </c>
       <c r="G177" t="str">
         <v>0.00</v>
       </c>
       <c r="H177" t="str">
-        <v>66951.36</v>
+        <v>64668.36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>